<commit_message>
feat: add post-write workbook validation step
</commit_message>
<xml_diff>
--- a/IOS_Master_Tracker_Filled_13.xlsx
+++ b/IOS_Master_Tracker_Filled_13.xlsx
@@ -1685,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BM37"/>
+  <dimension ref="A1:BN37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2050,6 +2050,11 @@
           <t>Valuation Label</t>
         </is>
       </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>Score Status</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="8" t="n">
@@ -2076,7 +2081,7 @@
         </is>
       </c>
       <c r="F2" s="8" t="n">
-        <v>186103906304</v>
+        <v>188288106496</v>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
@@ -2125,7 +2130,7 @@
         <v>1.85</v>
       </c>
       <c r="S2" s="8" t="n">
-        <v>31.50389117908067</v>
+        <v>31.87260344157299</v>
       </c>
       <c r="T2" s="8" t="n">
         <v>36.03169934056724</v>
@@ -2137,7 +2142,7 @@
         <v>0.05</v>
       </c>
       <c r="W2" s="8" t="n">
-        <v>2.377569345585877</v>
+        <v>2.350064878489226</v>
       </c>
       <c r="X2" s="8" t="n">
         <v>16</v>
@@ -2166,22 +2171,22 @@
         </is>
       </c>
       <c r="AH2" s="9" t="n">
-        <v>229.3533335282446</v>
+        <v>228.3150413406822</v>
       </c>
       <c r="AI2" s="10" t="n">
         <v>752</v>
       </c>
       <c r="AJ2" s="9" t="n">
-        <v>286.6916669103057</v>
+        <v>285.3938016758528</v>
       </c>
       <c r="AK2" s="11" t="n">
-        <v>-161.535330998854</v>
+        <v>-165.8081554488733</v>
       </c>
       <c r="AL2" s="8" t="n">
-        <v>4.59326171629291</v>
+        <v>4.363239954314882</v>
       </c>
       <c r="AM2" s="12" t="n">
-        <v>45932.61716292911</v>
+        <v>43632.39954314882</v>
       </c>
       <c r="AN2" s="8" t="inlineStr">
         <is>
@@ -2229,20 +2234,20 @@
         </is>
       </c>
       <c r="AW2" s="13" t="n">
-        <v>19.10000121763144</v>
+        <v>18.45000142035339</v>
       </c>
       <c r="AX2" s="13" t="n">
         <v>13.813758</v>
       </c>
       <c r="AY2" s="23" t="n">
-        <v>15.01003491676993</v>
+        <v>15.46849873581858</v>
       </c>
       <c r="AZ2" s="23" t="n">
         <v>1.61</v>
       </c>
       <c r="BA2" s="23" t="n"/>
       <c r="BB2" s="23" t="n">
-        <v>39.256542</v>
+        <v>41.116528</v>
       </c>
       <c r="BC2" s="23" t="n"/>
       <c r="BD2" s="23" t="n">
@@ -2270,6 +2275,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="8" t="n">
@@ -2296,7 +2306,7 @@
         </is>
       </c>
       <c r="F3" s="8" t="n">
-        <v>7444214841344</v>
+        <v>7369682583552</v>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
@@ -2312,7 +2322,7 @@
         <v>74</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>85.37205298601414</v>
+        <v>85.77298128093912</v>
       </c>
       <c r="K3" s="8" t="n">
         <v>95</v>
@@ -2345,7 +2355,7 @@
         <v>1.66</v>
       </c>
       <c r="S3" s="8" t="n">
-        <v>11.19837492367282</v>
+        <v>11.08716926315538</v>
       </c>
       <c r="T3" s="8" t="n">
         <v>45.36403694758384</v>
@@ -2357,7 +2367,7 @@
         <v>0.11</v>
       </c>
       <c r="W3" s="8" t="n">
-        <v>6.38848838513359</v>
+        <v>6.452565703131944</v>
       </c>
       <c r="X3" s="8" t="n">
         <v>6</v>
@@ -2386,22 +2396,22 @@
         </is>
       </c>
       <c r="AH3" s="9" t="n">
-        <v>2310.507247880147</v>
+        <v>2306.955761101446</v>
       </c>
       <c r="AI3" s="10" t="n">
         <v>1983</v>
       </c>
       <c r="AJ3" s="9" t="n">
-        <v>2888.134059850184</v>
+        <v>2883.694701376807</v>
       </c>
       <c r="AK3" s="11" t="n">
-        <v>28.76023213040434</v>
+        <v>29.36492205546269</v>
       </c>
       <c r="AL3" s="8" t="n">
-        <v>8.498507490158261</v>
+        <v>8.110830912442234</v>
       </c>
       <c r="AM3" s="12" t="n">
-        <v>84985.07490158261</v>
+        <v>81108.30912442233</v>
       </c>
       <c r="AN3" s="8" t="inlineStr">
         <is>
@@ -2449,20 +2459,20 @@
         </is>
       </c>
       <c r="AW3" s="13" t="n">
-        <v>136.039997015385</v>
+        <v>133.5299910824858</v>
       </c>
       <c r="AX3" s="13" t="n">
         <v>25</v>
       </c>
       <c r="AY3" s="23" t="n">
-        <v>21.23003572368556</v>
+        <v>21.59585637217709</v>
       </c>
       <c r="AZ3" s="23" t="n">
         <v>5.92</v>
       </c>
       <c r="BA3" s="23" t="n"/>
       <c r="BB3" s="23" t="n">
-        <v>15.1242285</v>
+        <v>15.254251</v>
       </c>
       <c r="BC3" s="23" t="n"/>
       <c r="BD3" s="23" t="n">
@@ -2490,6 +2500,11 @@
           <t>Undervalued</t>
         </is>
       </c>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="8" t="n">
@@ -2516,7 +2531,7 @@
         </is>
       </c>
       <c r="F4" s="8" t="n">
-        <v>1124334829568</v>
+        <v>1144093147136</v>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
@@ -2532,7 +2547,7 @@
         <v>94</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>69.98637920015651</v>
+        <v>68.795630807086</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>94</v>
@@ -2565,7 +2580,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="S4" s="8" t="n">
-        <v>7.829358020807081</v>
+        <v>7.963937346736105</v>
       </c>
       <c r="T4" s="8" t="n">
         <v>23.68743551054329</v>
@@ -2577,7 +2592,7 @@
         <v>0.29</v>
       </c>
       <c r="W4" s="8" t="n">
-        <v>4.593115510849442</v>
+        <v>4.515498326980259</v>
       </c>
       <c r="X4" s="8" t="n">
         <v>23</v>
@@ -2606,22 +2621,22 @@
         </is>
       </c>
       <c r="AH4" s="9" t="n">
-        <v>2080.374486953877</v>
+        <v>2077.508959149081</v>
       </c>
       <c r="AI4" s="10" t="n">
         <v>2476</v>
       </c>
       <c r="AJ4" s="9" t="n">
-        <v>2600.468108692347</v>
+        <v>2596.886198936351</v>
       </c>
       <c r="AK4" s="11" t="n">
-        <v>5.440101657831296</v>
+        <v>3.646143561282495</v>
       </c>
       <c r="AL4" s="8" t="n">
-        <v>6.966914195433777</v>
+        <v>6.505425375893696</v>
       </c>
       <c r="AM4" s="12" t="n">
-        <v>69669.14195433777</v>
+        <v>65054.25375893696</v>
       </c>
       <c r="AN4" s="8" t="inlineStr">
         <is>
@@ -2669,20 +2684,20 @@
         </is>
       </c>
       <c r="AW4" s="13" t="n">
-        <v>116.5399971526136</v>
+        <v>115.0800064057003</v>
       </c>
       <c r="AX4" s="13" t="n">
         <v>24.1328883</v>
       </c>
       <c r="AY4" s="23" t="n">
-        <v>22.31395322372015</v>
+        <v>22.56592108912367</v>
       </c>
       <c r="AZ4" s="23" t="n">
         <v>0.48</v>
       </c>
       <c r="BA4" s="23" t="n"/>
       <c r="BB4" s="23" t="n">
-        <v>21.100052</v>
+        <v>21.743134</v>
       </c>
       <c r="BC4" s="23" t="n"/>
       <c r="BD4" s="23" t="n">
@@ -2710,6 +2725,11 @@
           <t>Fair Value</t>
         </is>
       </c>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="8" t="n">
@@ -2736,7 +2756,7 @@
         </is>
       </c>
       <c r="F5" s="8" t="n">
-        <v>77266386944</v>
+        <v>78520582144</v>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
@@ -2784,7 +2804,9 @@
       <c r="R5" s="8" t="n">
         <v>1.2</v>
       </c>
-      <c r="S5" s="8" t="n"/>
+      <c r="S5" s="8" t="n">
+        <v/>
+      </c>
       <c r="T5" s="8" t="n">
         <v>13.77443749541119</v>
       </c>
@@ -2794,7 +2816,9 @@
       <c r="V5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="W5" s="8" t="n"/>
+      <c r="W5" s="8" t="n">
+        <v/>
+      </c>
       <c r="X5" s="8" t="n">
         <v>13</v>
       </c>
@@ -2822,22 +2846,22 @@
         </is>
       </c>
       <c r="AH5" s="9" t="n">
-        <v>374.6128220556247</v>
+        <v>384.5198705287766</v>
       </c>
       <c r="AI5" s="10" t="n">
         <v>1149</v>
       </c>
       <c r="AJ5" s="9" t="n">
-        <v>468.2660275695309</v>
+        <v>480.6498381609707</v>
       </c>
       <c r="AK5" s="11" t="n">
-        <v>-134.1831214388428</v>
+        <v>-131.8527775363122</v>
       </c>
       <c r="AL5" s="8" t="n">
-        <v>2.036692475707844</v>
+        <v>1.934698811770095</v>
       </c>
       <c r="AM5" s="12" t="n">
-        <v>20366.92475707844</v>
+        <v>19346.98811770095</v>
       </c>
       <c r="AN5" s="8" t="inlineStr">
         <is>
@@ -2888,17 +2912,17 @@
         <v>58.54000188976479</v>
       </c>
       <c r="AX5" s="13" t="n">
-        <v>10</v>
+        <v>13.044297</v>
       </c>
       <c r="AY5" s="23" t="n">
-        <v>7.999078024761375</v>
+        <v>8.210622448940395</v>
       </c>
       <c r="AZ5" s="23" t="n">
         <v>0.61</v>
       </c>
       <c r="BA5" s="23" t="n"/>
       <c r="BB5" s="23" t="n">
-        <v>18.73249</v>
+        <v>19.036556</v>
       </c>
       <c r="BC5" s="23" t="n"/>
       <c r="BD5" s="23" t="n">
@@ -2926,6 +2950,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN5" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="8" t="n">
@@ -2952,7 +2981,7 @@
         </is>
       </c>
       <c r="F6" s="8" t="n">
-        <v>745143926784</v>
+        <v>744956428288</v>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
@@ -3003,7 +3032,7 @@
         <v>1.04</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>30.89535713517239</v>
+        <v>30.88752018451047</v>
       </c>
       <c r="T6" s="8" t="n">
         <v>23.79630651498401</v>
@@ -3015,7 +3044,7 @@
         <v>0.06</v>
       </c>
       <c r="W6" s="8" t="n">
-        <v>2.108514370282366</v>
+        <v>2.109049354087837</v>
       </c>
       <c r="X6" s="8" t="n">
         <v>19.6</v>
@@ -3044,22 +3073,22 @@
         </is>
       </c>
       <c r="AH6" s="9" t="n">
-        <v>1580.947270717989</v>
+        <v>1575.45372227598</v>
       </c>
       <c r="AI6" s="10" t="n">
         <v>4683</v>
       </c>
       <c r="AJ6" s="9" t="n">
-        <v>1976.184088397486</v>
+        <v>1969.317152844974</v>
       </c>
       <c r="AK6" s="11" t="n">
-        <v>-141.3489729019957</v>
+        <v>-142.1296129529708</v>
       </c>
       <c r="AL6" s="15" t="n">
-        <v>3.973017437890814</v>
+        <v>3.774056323136255</v>
       </c>
       <c r="AM6" s="12" t="n">
-        <v>39730.17437890814</v>
+        <v>37740.56323136255</v>
       </c>
       <c r="AN6" s="8" t="inlineStr">
         <is>
@@ -3107,20 +3136,20 @@
         </is>
       </c>
       <c r="AW6" s="13" t="n">
-        <v>118.6999967397632</v>
+        <v>115.9000036459536</v>
       </c>
       <c r="AX6" s="13" t="n">
         <v>18.14655820438004</v>
       </c>
       <c r="AY6" s="23" t="n">
-        <v>16.64856013814226</v>
+        <v>16.9915198692405</v>
       </c>
       <c r="AZ6" s="23" t="n">
         <v>0.9</v>
       </c>
       <c r="BA6" s="23" t="n"/>
       <c r="BB6" s="23" t="n">
-        <v>40.18113</v>
+        <v>41.1415</v>
       </c>
       <c r="BC6" s="23" t="n"/>
       <c r="BD6" s="23" t="n">
@@ -3148,6 +3177,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN6" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="8" t="n">
@@ -3174,7 +3208,7 @@
         </is>
       </c>
       <c r="F7" s="8" t="n">
-        <v>247531388928</v>
+        <v>254148067328</v>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
@@ -3222,7 +3256,9 @@
       <c r="R7" s="8" t="n">
         <v>4.07</v>
       </c>
-      <c r="S7" s="8" t="n"/>
+      <c r="S7" s="8" t="n">
+        <v/>
+      </c>
       <c r="T7" s="8" t="n">
         <v>19.11976068675267</v>
       </c>
@@ -3232,7 +3268,9 @@
       <c r="V7" s="8" t="n">
         <v>0.08</v>
       </c>
-      <c r="W7" s="8" t="n"/>
+      <c r="W7" s="8" t="n">
+        <v/>
+      </c>
       <c r="X7" s="8" t="n">
         <v>28</v>
       </c>
@@ -3269,13 +3307,13 @@
         <v>241.3281220099968</v>
       </c>
       <c r="AK7" s="11" t="n">
-        <v>-806.8565991282787</v>
+        <v>-831.0974540741339</v>
       </c>
       <c r="AL7" s="15" t="n">
-        <v>2.530550537048101</v>
+        <v>2.403825405919271</v>
       </c>
       <c r="AM7" s="12" t="n">
-        <v>25305.50537048101</v>
+        <v>24038.25405919271</v>
       </c>
       <c r="AN7" s="8" t="inlineStr">
         <is>
@@ -3336,7 +3374,7 @@
       </c>
       <c r="BA7" s="23" t="n"/>
       <c r="BB7" s="23" t="n">
-        <v>50.20647</v>
+        <v>51.54852</v>
       </c>
       <c r="BC7" s="23" t="n"/>
       <c r="BD7" s="23" t="n">
@@ -3364,6 +3402,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN7" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="8" t="n">
@@ -3390,7 +3433,7 @@
         </is>
       </c>
       <c r="F8" s="8" t="n">
-        <v>1524184252416</v>
+        <v>1532361572352</v>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
@@ -3439,7 +3482,7 @@
         <v>2.05</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>63.41098973088238</v>
+        <v>63.75223036501346</v>
       </c>
       <c r="T8" s="8" t="n">
         <v>27.86673053960043</v>
@@ -3451,7 +3494,7 @@
         <v>0.003</v>
       </c>
       <c r="W8" s="8" t="n">
-        <v>0.9756511660565308</v>
+        <v>0.9704288888014504</v>
       </c>
       <c r="X8" s="8" t="n">
         <v>13</v>
@@ -3480,22 +3523,22 @@
         </is>
       </c>
       <c r="AH8" s="9" t="n">
-        <v>739.3485718840109</v>
+        <v>756.6900032601275</v>
       </c>
       <c r="AI8" s="10" t="n">
         <v>5478</v>
       </c>
       <c r="AJ8" s="9" t="n">
-        <v>924.1857148550135</v>
+        <v>945.8625040751592</v>
       </c>
       <c r="AK8" s="11" t="n">
-        <v>-494.9561772725091</v>
+        <v>-484.4401248789474</v>
       </c>
       <c r="AL8" s="15" t="n">
-        <v>4.435525134546993</v>
+        <v>4.213402518906062</v>
       </c>
       <c r="AM8" s="12" t="n">
-        <v>44355.25134546993</v>
+        <v>42134.02518906062</v>
       </c>
       <c r="AN8" s="8" t="inlineStr">
         <is>
@@ -3546,17 +3589,17 @@
         <v>85.36000935179952</v>
       </c>
       <c r="AX8" s="13" t="n">
-        <v>10</v>
+        <v>10.9602055</v>
       </c>
       <c r="AY8" s="23" t="n">
-        <v>10.82691793410278</v>
+        <v>11.08086344980271</v>
       </c>
       <c r="AZ8" s="23" t="n">
         <v>1.21</v>
       </c>
       <c r="BA8" s="23" t="n"/>
       <c r="BB8" s="23" t="n">
-        <v>64.41540999999999</v>
+        <v>64.76101</v>
       </c>
       <c r="BC8" s="23" t="n"/>
       <c r="BD8" s="23" t="n">
@@ -3584,6 +3627,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="8" t="n">
@@ -3610,7 +3658,7 @@
         </is>
       </c>
       <c r="F9" s="8" t="n">
-        <v>209980358656</v>
+        <v>218085507072</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -3659,7 +3707,7 @@
         <v>2.49</v>
       </c>
       <c r="S9" s="8" t="n">
-        <v>156.9499773507318</v>
+        <v>162.9017242287838</v>
       </c>
       <c r="T9" s="8" t="n">
         <v>11.43100972906209</v>
@@ -3671,7 +3719,7 @@
         <v>0.3</v>
       </c>
       <c r="W9" s="8" t="n">
-        <v>0.2961596810553887</v>
+        <v>0.2853392464315615</v>
       </c>
       <c r="X9" s="8" t="n">
         <v>29.6</v>
@@ -3709,13 +3757,13 @@
         <v>442.3257396743983</v>
       </c>
       <c r="AK9" s="11" t="n">
-        <v>-1443.319637022497</v>
+        <v>-1502.891119386143</v>
       </c>
       <c r="AL9" s="15" t="n">
-        <v>1.200967875368491</v>
+        <v>1.140825701063165</v>
       </c>
       <c r="AM9" s="12" t="n">
-        <v>12009.67875368491</v>
+        <v>11408.25701063165</v>
       </c>
       <c r="AN9" s="8" t="inlineStr">
         <is>
@@ -3774,7 +3822,7 @@
       <c r="AZ9" s="23" t="n"/>
       <c r="BA9" s="23" t="n"/>
       <c r="BB9" s="23" t="n">
-        <v>221.42393</v>
+        <v>229.97081</v>
       </c>
       <c r="BC9" s="23" t="n"/>
       <c r="BD9" s="23" t="n">
@@ -3802,6 +3850,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN9" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="8" t="n">
@@ -3828,7 +3881,7 @@
         </is>
       </c>
       <c r="F10" s="8" t="n">
-        <v>437135409152</v>
+        <v>436117504000</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
@@ -3877,7 +3930,7 @@
         <v>1.13</v>
       </c>
       <c r="S10" s="8" t="n">
-        <v>38.38724894030482</v>
+        <v>38.3059810144268</v>
       </c>
       <c r="T10" s="8" t="n">
         <v>10.22446814323704</v>
@@ -3889,7 +3942,7 @@
         <v>0.1</v>
       </c>
       <c r="W10" s="8" t="n">
-        <v>2.509942511870562</v>
+        <v>2.515267472010232</v>
       </c>
       <c r="X10" s="8" t="n">
         <v>-0.1</v>
@@ -3918,22 +3971,22 @@
         </is>
       </c>
       <c r="AH10" s="9" t="n">
-        <v>435.7429123304599</v>
+        <v>427.9494491855152</v>
       </c>
       <c r="AI10" s="10" t="n">
         <v>1325</v>
       </c>
       <c r="AJ10" s="9" t="n">
-        <v>544.6786404130748</v>
+        <v>534.936811481894</v>
       </c>
       <c r="AK10" s="11" t="n">
-        <v>-128.6485842469443</v>
+        <v>-132.2704239698888</v>
       </c>
       <c r="AL10" s="15" t="n">
-        <v>0.7221262421359587</v>
+        <v>0.685963541021522</v>
       </c>
       <c r="AM10" s="12" t="n">
-        <v>7221.262421359587</v>
+        <v>6859.63541021522</v>
       </c>
       <c r="AN10" s="8" t="inlineStr">
         <is>
@@ -3981,20 +4034,20 @@
         </is>
       </c>
       <c r="AW10" s="13" t="n">
-        <v>25.59999973688775</v>
+        <v>23.0400014478578</v>
       </c>
       <c r="AX10" s="13" t="n">
         <v>10.48834958223998</v>
       </c>
       <c r="AY10" s="23" t="n">
-        <v>21.27650939113574</v>
+        <v>23.21774355390165</v>
       </c>
       <c r="AZ10" s="23" t="n">
         <v>0.97</v>
       </c>
       <c r="BA10" s="23" t="n"/>
       <c r="BB10" s="23" t="n">
-        <v>48.648438</v>
+        <v>53.927948</v>
       </c>
       <c r="BC10" s="23" t="n"/>
       <c r="BD10" s="23" t="n">
@@ -4022,6 +4075,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN10" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="8" t="n">
@@ -4048,7 +4106,7 @@
         </is>
       </c>
       <c r="F11" s="8" t="n">
-        <v>242343772160</v>
+        <v>249297567744</v>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
@@ -4097,7 +4155,7 @@
         <v>1.66</v>
       </c>
       <c r="S11" s="8" t="n">
-        <v>50.66506161779093</v>
+        <v>52.10549165990518</v>
       </c>
       <c r="T11" s="8" t="n">
         <v>19.41870698690816</v>
@@ -4109,7 +4167,7 @@
         <v>0.4</v>
       </c>
       <c r="W11" s="8" t="n">
-        <v>-0.2062706704437527</v>
+        <v>-0.2005684217738135</v>
       </c>
       <c r="X11" s="8" t="n">
         <v>37</v>
@@ -4138,22 +4196,22 @@
         </is>
       </c>
       <c r="AH11" s="9" t="n">
-        <v>904.6808310954592</v>
+        <v>902.8731126065013</v>
       </c>
       <c r="AI11" s="10" t="n">
         <v>18944</v>
       </c>
       <c r="AJ11" s="9" t="n">
-        <v>1130.851038869324</v>
+        <v>1128.591390758127</v>
       </c>
       <c r="AK11" s="11" t="n">
-        <v>-1570.334938091057</v>
+        <v>-1621.703723696431</v>
       </c>
       <c r="AL11" s="15" t="n">
-        <v>3.07035961182777</v>
+        <v>2.916601874637739</v>
       </c>
       <c r="AM11" s="12" t="n">
-        <v>30703.5961182777</v>
+        <v>29166.01874637738</v>
       </c>
       <c r="AN11" s="8" t="inlineStr">
         <is>
@@ -4207,14 +4265,14 @@
         <v>10</v>
       </c>
       <c r="AY11" s="23" t="n">
-        <v>3.977108528062615</v>
+        <v>3.980922013256178</v>
       </c>
       <c r="AZ11" s="23" t="n">
         <v>0.18</v>
       </c>
       <c r="BA11" s="23" t="n"/>
       <c r="BB11" s="23" t="n">
-        <v>66.62787</v>
+        <v>68.53968</v>
       </c>
       <c r="BC11" s="23" t="n"/>
       <c r="BD11" s="23" t="n">
@@ -4242,6 +4300,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN11" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="8" t="n">
@@ -4268,7 +4331,7 @@
         </is>
       </c>
       <c r="F12" s="8" t="n">
-        <v>111762382848</v>
+        <v>113613684736</v>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
@@ -4317,7 +4380,7 @@
         <v>1.85</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>26.28249478015705</v>
+        <v>26.713862743435</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>14.79510631746486</v>
@@ -4329,7 +4392,7 @@
         <v>0.12</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>1.726116120577604</v>
+        <v>1.698243281577643</v>
       </c>
       <c r="X12" s="8" t="n">
         <v>17.5</v>
@@ -4367,13 +4430,13 @@
         <v>195.9127694974635</v>
       </c>
       <c r="AK12" s="11" t="n">
-        <v>-154.2202845059819</v>
+        <v>-158.4313423258279</v>
       </c>
       <c r="AL12" s="15" t="n">
-        <v>1.953014624127069</v>
+        <v>1.855211386959662</v>
       </c>
       <c r="AM12" s="12" t="n">
-        <v>19530.14624127069</v>
+        <v>18552.11386959662</v>
       </c>
       <c r="AN12" s="8" t="inlineStr">
         <is>
@@ -4434,7 +4497,7 @@
       </c>
       <c r="BA12" s="23" t="n"/>
       <c r="BB12" s="23" t="n">
-        <v>32.809616</v>
+        <v>33.353096</v>
       </c>
       <c r="BC12" s="23" t="n"/>
       <c r="BD12" s="23" t="n">
@@ -4462,6 +4525,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN12" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="8" t="n">
@@ -4488,7 +4556,7 @@
         </is>
       </c>
       <c r="F13" s="8" t="n">
-        <v>9386615373824</v>
+        <v>9464152326144</v>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
@@ -4547,7 +4615,7 @@
         <v>1.33</v>
       </c>
       <c r="W13" s="8" t="n">
-        <v>2.923140132205341</v>
+        <v>2.901026988552449</v>
       </c>
       <c r="X13" s="8" t="n">
         <v>5.2</v>
@@ -4576,16 +4644,16 @@
         </is>
       </c>
       <c r="AH13" s="9" t="n">
-        <v>728.2310545303662</v>
+        <v>759.4077480976221</v>
       </c>
       <c r="AI13" s="10" t="n">
         <v>1040</v>
       </c>
       <c r="AJ13" s="9" t="n">
-        <v>910.2888181629578</v>
+        <v>949.2596851220275</v>
       </c>
       <c r="AK13" s="11" t="n">
-        <v>-11.71179736692722</v>
+        <v>-8.010486073491839</v>
       </c>
       <c r="AL13" s="15" t="n">
         <v>0.282075058945176</v>
@@ -4642,17 +4710,17 @@
         <v>91.15000343710916</v>
       </c>
       <c r="AX13" s="13" t="n">
-        <v>10</v>
+        <v>12.7778112</v>
       </c>
       <c r="AY13" s="23" t="n">
-        <v>9.986712212429596</v>
+        <v>10.41425875065307</v>
       </c>
       <c r="AZ13" s="23" t="n">
         <v>1.67</v>
       </c>
       <c r="BA13" s="23" t="n"/>
       <c r="BB13" s="23" t="n">
-        <v>11.156336</v>
+        <v>11.248492</v>
       </c>
       <c r="BC13" s="23" t="n"/>
       <c r="BD13" s="23" t="n">
@@ -4680,6 +4748,11 @@
           <t>Overvalued</t>
         </is>
       </c>
+      <c r="BN13" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="8" t="n">
@@ -4706,7 +4779,7 @@
         </is>
       </c>
       <c r="F14" s="8" t="n">
-        <v>4068344332288</v>
+        <v>4070739542016</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -4754,7 +4827,9 @@
       <c r="R14" s="8" t="n">
         <v>4.64</v>
       </c>
-      <c r="S14" s="8" t="n"/>
+      <c r="S14" s="8" t="n">
+        <v/>
+      </c>
       <c r="T14" s="8" t="n">
         <v>32.30592880341336</v>
       </c>
@@ -4764,7 +4839,9 @@
       <c r="V14" s="8" t="n">
         <v>1.5</v>
       </c>
-      <c r="W14" s="8" t="n"/>
+      <c r="W14" s="8" t="n">
+        <v/>
+      </c>
       <c r="X14" s="8" t="n">
         <v>17</v>
       </c>
@@ -4801,7 +4878,7 @@
         <v>1199.185730484497</v>
       </c>
       <c r="AK14" s="11" t="n">
-        <v>-282.4595209406798</v>
+        <v>-282.6846737198836</v>
       </c>
       <c r="AL14" s="15">
         <f>IF(H14="Fail","Not Eligible (Failed Gate)",IF(J14="","Pending Score",IF(J14&gt;=90,"10%",IF(J14&gt;=80,"7.5%",IF(J14&gt;=70,"5%","Watchlist only")))))</f>
@@ -4870,7 +4947,7 @@
       </c>
       <c r="BA14" s="23" t="n"/>
       <c r="BB14" s="23" t="n">
-        <v>80.33631</v>
+        <v>80.383606</v>
       </c>
       <c r="BC14" s="23" t="n"/>
       <c r="BD14" s="23" t="n">
@@ -4898,6 +4975,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN14" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="8" t="n">
@@ -4924,7 +5006,7 @@
         </is>
       </c>
       <c r="F15" s="8" t="n">
-        <v>1265662951424</v>
+        <v>1255564640256</v>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
@@ -4973,7 +5055,7 @@
         <v>2.66</v>
       </c>
       <c r="S15" s="8" t="n">
-        <v>16.80694042182488</v>
+        <v>16.67025325540411</v>
       </c>
       <c r="T15" s="8" t="n">
         <v>15.99527878445324</v>
@@ -4985,7 +5067,7 @@
         <v>0.1</v>
       </c>
       <c r="W15" s="8" t="n">
-        <v>4.41039576560739</v>
+        <v>4.446558653522701</v>
       </c>
       <c r="X15" s="8" t="n">
         <v>8.460000000000001</v>
@@ -5014,22 +5096,22 @@
         </is>
       </c>
       <c r="AH15" s="9" t="n">
-        <v>757.5632469167359</v>
+        <v>661.6785928249716</v>
       </c>
       <c r="AI15" s="10" t="n">
         <v>1410</v>
       </c>
       <c r="AJ15" s="9" t="n">
-        <v>946.9540586459199</v>
+        <v>827.0982410312145</v>
       </c>
       <c r="AK15" s="11" t="n">
-        <v>-50.88377170515401</v>
+        <v>-71.37021089934925</v>
       </c>
       <c r="AL15" s="15" t="n">
-        <v>2.861640579656076</v>
+        <v>2.718335092414743</v>
       </c>
       <c r="AM15" s="12" t="n">
-        <v>28616.40579656076</v>
+        <v>27183.35092414743</v>
       </c>
       <c r="AN15" s="8" t="inlineStr">
         <is>
@@ -5077,20 +5159,20 @@
         </is>
       </c>
       <c r="AW15" s="13" t="n">
-        <v>54.13999705958582</v>
+        <v>53.43999716474687</v>
       </c>
       <c r="AX15" s="13" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AY15" s="23" t="n">
-        <v>17.49083964990617</v>
+        <v>15.47713774384758</v>
       </c>
       <c r="AZ15" s="23" t="n">
         <v>3.52</v>
       </c>
       <c r="BA15" s="23" t="n"/>
       <c r="BB15" s="23" t="n">
-        <v>26.39084</v>
+        <v>26.523205</v>
       </c>
       <c r="BC15" s="23" t="n"/>
       <c r="BD15" s="23" t="n">
@@ -5118,6 +5200,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN15" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="8" t="n">
@@ -5144,7 +5231,7 @@
         </is>
       </c>
       <c r="F16" s="8" t="n">
-        <v>5354475749376</v>
+        <v>5411980705792</v>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
@@ -5193,7 +5280,7 @@
         <v>2.5</v>
       </c>
       <c r="S16" s="8" t="n">
-        <v>24.55781444341955</v>
+        <v>24.77024054459141</v>
       </c>
       <c r="T16" s="8" t="n">
         <v>12.51375743928715</v>
@@ -5205,7 +5292,7 @@
         <v>1.12</v>
       </c>
       <c r="W16" s="8" t="n">
-        <v>1.794808523081884</v>
+        <v>1.77941649746865</v>
       </c>
       <c r="X16" s="8" t="n">
         <v>12</v>
@@ -5234,22 +5321,22 @@
         </is>
       </c>
       <c r="AH16" s="9" t="n">
-        <v>1389.36895284642</v>
+        <v>1381.490184242162</v>
       </c>
       <c r="AI16" s="10" t="n">
         <v>3693</v>
       </c>
       <c r="AJ16" s="9" t="n">
-        <v>1736.711191058025</v>
+        <v>1726.862730302702</v>
       </c>
       <c r="AK16" s="11" t="n">
-        <v>-124.1074981286259</v>
+        <v>-127.8061788565224</v>
       </c>
       <c r="AL16" s="15" t="n">
-        <v>0.03171664116764113</v>
+        <v>0.03012833243715284</v>
       </c>
       <c r="AM16" s="12" t="n">
-        <v>317.1664116764113</v>
+        <v>301.2833243715284</v>
       </c>
       <c r="AN16" s="8" t="inlineStr">
         <is>
@@ -5297,20 +5384,20 @@
         </is>
       </c>
       <c r="AW16" s="13" t="n">
-        <v>116.9599957207925</v>
+        <v>114.0400031424125</v>
       </c>
       <c r="AX16" s="13" t="n">
         <v>12.0206624909</v>
       </c>
       <c r="AY16" s="23" t="n">
-        <v>14.84876189345096</v>
+        <v>15.14260549195635</v>
       </c>
       <c r="AZ16" s="23" t="n">
         <v>0.95</v>
       </c>
       <c r="BA16" s="23" t="n"/>
       <c r="BB16" s="23" t="n">
-        <v>33.27719</v>
+        <v>34.49579</v>
       </c>
       <c r="BC16" s="23" t="n"/>
       <c r="BD16" s="23" t="n">
@@ -5338,6 +5425,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN16" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="8" t="n">
@@ -5364,7 +5456,7 @@
         </is>
       </c>
       <c r="F17" s="8" t="n">
-        <v>108983336960</v>
+        <v>115584335872</v>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
@@ -5412,7 +5504,9 @@
       <c r="R17" s="8" t="n">
         <v>1.99</v>
       </c>
-      <c r="S17" s="8" t="n"/>
+      <c r="S17" s="8" t="n">
+        <v/>
+      </c>
       <c r="T17" s="8" t="n">
         <v>15.64988464815957</v>
       </c>
@@ -5422,7 +5516,9 @@
       <c r="V17" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="W17" s="8" t="n"/>
+      <c r="W17" s="8" t="n">
+        <v/>
+      </c>
       <c r="X17" s="8" t="n">
         <v>18.4</v>
       </c>
@@ -5450,22 +5546,22 @@
         </is>
       </c>
       <c r="AH17" s="9" t="n">
-        <v>85.33777552403239</v>
+        <v>86.50060204353008</v>
       </c>
       <c r="AI17" s="10" t="n">
         <v>1800</v>
       </c>
       <c r="AJ17" s="9" t="n">
-        <v>106.6722194050405</v>
+        <v>108.1257525544126</v>
       </c>
       <c r="AK17" s="11" t="n">
-        <v>-1429.170396095576</v>
+        <v>-1499.988864012211</v>
       </c>
       <c r="AL17" s="15" t="n">
-        <v>1.438642286038537</v>
+        <v>1.36659783180749</v>
       </c>
       <c r="AM17" s="12" t="n">
-        <v>14386.42286038537</v>
+        <v>13665.9783180749</v>
       </c>
       <c r="AN17" s="8" t="inlineStr">
         <is>
@@ -5513,18 +5609,18 @@
         </is>
       </c>
       <c r="AW17" s="13" t="n">
-        <v>16.88999942636956</v>
+        <v>16.79999844624292</v>
       </c>
       <c r="AX17" s="13" t="n">
-        <v>10</v>
+        <v>16.943</v>
       </c>
       <c r="AY17" s="23" t="n">
-        <v>6.315702747486116</v>
+        <v>6.436056699667416</v>
       </c>
       <c r="AZ17" s="23" t="n"/>
       <c r="BA17" s="23" t="n"/>
       <c r="BB17" s="23" t="n">
-        <v>96.57786</v>
+        <v>102.9762</v>
       </c>
       <c r="BC17" s="23" t="n"/>
       <c r="BD17" s="23" t="n">
@@ -5552,6 +5648,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN17" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="8" t="n">
@@ -5578,7 +5679,7 @@
         </is>
       </c>
       <c r="F18" s="8" t="n">
-        <v>1430238527488</v>
+        <v>1438822170624</v>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
@@ -5627,7 +5728,7 @@
         <v>3.84</v>
       </c>
       <c r="S18" s="8" t="n">
-        <v>98.99425887145991</v>
+        <v>99.58818808245054</v>
       </c>
       <c r="T18" s="8" t="n">
         <v>14.71374988564633</v>
@@ -5639,7 +5740,7 @@
         <v>0.1</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>-0.05263876252079894</v>
+        <v>-0.05232483273360754</v>
       </c>
       <c r="X18" s="8" t="n">
         <v>25</v>
@@ -5677,13 +5778,13 @@
         <v>41.38406487047407</v>
       </c>
       <c r="AK18" s="11" t="n">
-        <v>-2094.322870027913</v>
+        <v>-2107.49219019271</v>
       </c>
       <c r="AL18" s="15" t="n">
-        <v>1.98668124475437</v>
+        <v>1.887192047614539</v>
       </c>
       <c r="AM18" s="12" t="n">
-        <v>19866.8124475437</v>
+        <v>18871.92047614539</v>
       </c>
       <c r="AN18" s="8" t="inlineStr">
         <is>
@@ -5744,7 +5845,7 @@
       </c>
       <c r="BA18" s="23" t="n"/>
       <c r="BB18" s="23" t="n">
-        <v>117.325584</v>
+        <v>118.02972</v>
       </c>
       <c r="BC18" s="23" t="n"/>
       <c r="BD18" s="23" t="n">
@@ -5772,6 +5873,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN18" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="8" t="n">
@@ -5798,7 +5904,7 @@
         </is>
       </c>
       <c r="F19" s="8" t="n">
-        <v>95095472128</v>
+        <v>96507510784</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
@@ -5855,7 +5961,7 @@
         <v>0.9</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>-5.511652749169317</v>
+        <v>-5.454949061932505</v>
       </c>
       <c r="X19" s="8" t="n">
         <v>-88</v>
@@ -5950,7 +6056,7 @@
         <v/>
       </c>
       <c r="AX19" s="13" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AY19" s="23">
         <f>IFERROR(IF(OR(T19="",T19=0,AW19="N/A",T19-AX19&lt;3),"N/A",ROUND((1-(AX19/T19))*100/(Dashboard!$B$14-AX19),1)),"N/A")</f>
@@ -5982,6 +6088,11 @@
           <t>Avoid</t>
         </is>
       </c>
+      <c r="BN19" t="inlineStr">
+        <is>
+          <t>Confirmed Weak Fundamentals</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="8" t="n">
@@ -6008,7 +6119,7 @@
         </is>
       </c>
       <c r="F20" s="8" t="n">
-        <v>257972961280</v>
+        <v>259950559232</v>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
@@ -6057,7 +6168,7 @@
         <v>0.57</v>
       </c>
       <c r="S20" s="8" t="n">
-        <v>33.0898493019063</v>
+        <v>33.2404162852492</v>
       </c>
       <c r="T20" s="8" t="n">
         <v>9.859652881090113</v>
@@ -6069,7 +6180,7 @@
         <v>0.65</v>
       </c>
       <c r="W20" s="8" t="n">
-        <v>-9.370658253868001</v>
+        <v>-9.328212583720113</v>
       </c>
       <c r="X20" s="8" t="n">
         <v>42.3</v>
@@ -6174,7 +6285,7 @@
       </c>
       <c r="BA20" s="23" t="n"/>
       <c r="BB20" s="23" t="n">
-        <v>44.815952</v>
+        <v>45.15951</v>
       </c>
       <c r="BC20" s="23" t="n"/>
       <c r="BD20" s="23" t="n">
@@ -6197,6 +6308,11 @@
           <t>Avoid</t>
         </is>
       </c>
+      <c r="BN20" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="8" t="n">
@@ -6223,7 +6339,7 @@
         </is>
       </c>
       <c r="F21" s="8" t="n">
-        <v>13158268928</v>
+        <v>13353916416</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
@@ -6272,7 +6388,7 @@
         <v>5.08</v>
       </c>
       <c r="S21" s="8" t="n">
-        <v>21.99614283450168</v>
+        <v>22.29429505638525</v>
       </c>
       <c r="T21" s="8" t="n">
         <v>8.622202272866382</v>
@@ -6284,7 +6400,7 @@
         <v>0.2</v>
       </c>
       <c r="W21" s="8" t="n">
-        <v>2.526696077255663</v>
+        <v>2.49290536767938</v>
       </c>
       <c r="X21" s="8" t="n">
         <v>2</v>
@@ -6313,22 +6429,22 @@
         </is>
       </c>
       <c r="AH21" s="9" t="n">
-        <v>204.7910955117359</v>
+        <v>202.8668495016184</v>
       </c>
       <c r="AI21" s="10" t="n">
         <v>495</v>
       </c>
       <c r="AJ21" s="9" t="n">
-        <v>255.9888693896698</v>
+        <v>253.583561877023</v>
       </c>
       <c r="AK21" s="11" t="n">
-        <v>-85.2228970464502</v>
+        <v>-89.75993413696153</v>
       </c>
       <c r="AL21" s="15" t="n">
-        <v>1.193165273398202</v>
+        <v>1.133413838476798</v>
       </c>
       <c r="AM21" s="12" t="n">
-        <v>11931.65273398202</v>
+        <v>11334.13838476798</v>
       </c>
       <c r="AN21" s="8" t="inlineStr">
         <is>
@@ -6376,18 +6492,18 @@
         </is>
       </c>
       <c r="AW21" s="13" t="n">
-        <v>15.23999937516485</v>
+        <v>14.65000017049044</v>
       </c>
       <c r="AX21" s="13" t="n">
         <v>10</v>
       </c>
       <c r="AY21" s="23" t="n">
-        <v>16.79716990745865</v>
+        <v>17.30945814860225</v>
       </c>
       <c r="AZ21" s="23" t="n"/>
       <c r="BA21" s="23" t="n"/>
       <c r="BB21" s="23" t="n">
-        <v>31.112206</v>
+        <v>32.846416</v>
       </c>
       <c r="BC21" s="23" t="n"/>
       <c r="BD21" s="23" t="n">
@@ -6415,6 +6531,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN21" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="8" t="n">
@@ -6441,7 +6562,7 @@
         </is>
       </c>
       <c r="F22" s="8" t="n">
-        <v>46791028736</v>
+        <v>47571521536</v>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
@@ -6490,7 +6611,7 @@
         <v>6.97</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>42.58236185493899</v>
+        <v>42.97436206387377</v>
       </c>
       <c r="T22" s="8" t="n">
         <v>8.870267856766871</v>
@@ -6502,7 +6623,7 @@
         <v>1.2</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>1.299075226018463</v>
+        <v>1.287225422192071</v>
       </c>
       <c r="X22" s="8" t="n">
         <v>7.5</v>
@@ -6531,16 +6652,16 @@
         </is>
       </c>
       <c r="AH22" s="9" t="n">
-        <v>64.33319872860064</v>
+        <v>64.26943015681294</v>
       </c>
       <c r="AI22" s="10" t="n">
         <v>230</v>
       </c>
       <c r="AJ22" s="9" t="n">
-        <v>80.41649841075079</v>
+        <v>80.33678769601617</v>
       </c>
       <c r="AK22" s="11" t="n">
-        <v>-188.5104482104419</v>
+        <v>-193.6139305103147</v>
       </c>
       <c r="AL22" s="15">
         <f>IF(H22="Fail","Not Eligible (Failed Gate)",IF(J22="","Pending Score",IF(J22&gt;=90,"10%",IF(J22&gt;=80,"7.5%",IF(J22&gt;=70,"5%","Watchlist only")))))</f>
@@ -6596,18 +6717,18 @@
         </is>
       </c>
       <c r="AW22" s="13" t="n">
-        <v>3.450000089610392</v>
+        <v>3.429999965100899</v>
       </c>
       <c r="AX22" s="13" t="n">
         <v>8.972</v>
       </c>
       <c r="AY22" s="23" t="n">
-        <v>23.30912997413066</v>
+        <v>23.42180399300763</v>
       </c>
       <c r="AZ22" s="23" t="n"/>
       <c r="BA22" s="23" t="n"/>
       <c r="BB22" s="23" t="n">
-        <v>67.249275</v>
+        <v>68.76967999999999</v>
       </c>
       <c r="BC22" s="23" t="n"/>
       <c r="BD22" s="23" t="n">
@@ -6635,6 +6756,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN22" t="inlineStr">
+        <is>
+          <t>Confirmed Weak Fundamentals</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="8" t="n">
@@ -6661,7 +6787,7 @@
         </is>
       </c>
       <c r="F23" s="8" t="n">
-        <v>1331921027072</v>
+        <v>1333406072832</v>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
@@ -6720,7 +6846,7 @@
         <v>8.25</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>-0.4097501574392843</v>
+        <v>-0.4096986662627712</v>
       </c>
       <c r="X23" s="8" t="n">
         <v>10</v>
@@ -6749,16 +6875,16 @@
         </is>
       </c>
       <c r="AH23" s="9" t="n">
-        <v>233.4882156117897</v>
+        <v>228.9944597100921</v>
       </c>
       <c r="AI23" s="10" t="n">
         <v>423</v>
       </c>
       <c r="AJ23" s="9" t="n">
-        <v>291.8602695147371</v>
+        <v>286.2430746376151</v>
       </c>
       <c r="AK23" s="11" t="n">
-        <v>-38.28535164140275</v>
+        <v>-41.15625347845671</v>
       </c>
       <c r="AL23" s="15" t="n">
         <v>0.05722510500731424</v>
@@ -6812,20 +6938,20 @@
         </is>
       </c>
       <c r="AW23" s="13" t="n">
-        <v>78.49999960127602</v>
+        <v>76.67999987095064</v>
       </c>
       <c r="AX23" s="13" t="n">
         <v>16.12516180932</v>
       </c>
       <c r="AY23" s="23" t="n">
-        <v>3.717965216748244</v>
+        <v>3.732956111601657</v>
       </c>
       <c r="AZ23" s="23" t="n">
         <v>3.82</v>
       </c>
       <c r="BA23" s="23" t="n"/>
       <c r="BB23" s="23" t="n">
-        <v>5.1414013</v>
+        <v>5.269301</v>
       </c>
       <c r="BC23" s="23" t="n"/>
       <c r="BD23" s="23" t="n">
@@ -6853,6 +6979,11 @@
           <t>Overvalued</t>
         </is>
       </c>
+      <c r="BN23" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="8" t="n">
@@ -6879,7 +7010,7 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>3516395159552</v>
+        <v>3530177642496</v>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
@@ -6895,7 +7026,7 @@
         <v>77</v>
       </c>
       <c r="J24" s="15" t="n">
-        <v>46.97031688616686</v>
+        <v>37.23237914388618</v>
       </c>
       <c r="K24" s="8" t="n">
         <v>80</v>
@@ -6928,7 +7059,7 @@
         <v>2.71</v>
       </c>
       <c r="S24" s="8" t="n">
-        <v>13.82120228583574</v>
+        <v>13.87504949102851</v>
       </c>
       <c r="T24" s="8" t="n">
         <v>28.39112472627043</v>
@@ -6940,7 +7071,7 @@
         <v>0.03</v>
       </c>
       <c r="W24" s="8" t="n">
-        <v>4.602376673186018</v>
+        <v>4.584515466906663</v>
       </c>
       <c r="X24" s="8" t="n">
         <v>9.869999999999999</v>
@@ -6969,22 +7100,22 @@
         </is>
       </c>
       <c r="AH24" s="9" t="n">
-        <v>163.9756645962809</v>
+        <v>143.3293811775836</v>
       </c>
       <c r="AI24" s="10" t="n">
         <v>289</v>
       </c>
       <c r="AJ24" s="9" t="n">
-        <v>204.9695807453511</v>
+        <v>179.1617264719795</v>
       </c>
       <c r="AK24" s="11" t="n">
-        <v>-36.92275652779535</v>
+        <v>-57.26015011585921</v>
       </c>
       <c r="AL24" s="15" t="n">
-        <v>4.675740782965478</v>
+        <v>3.520753589232069</v>
       </c>
       <c r="AM24" s="12" t="n">
-        <v>46757.40782965478</v>
+        <v>35207.53589232069</v>
       </c>
       <c r="AN24" s="8" t="inlineStr">
         <is>
@@ -7032,20 +7163,20 @@
         </is>
       </c>
       <c r="AW24" s="13" t="n">
-        <v>16.51999979515553</v>
+        <v>16.04999920818105</v>
       </c>
       <c r="AX24" s="13" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AY24" s="23" t="n">
-        <v>12.40735960928275</v>
+        <v>11.16272439077754</v>
       </c>
       <c r="AZ24" s="23" t="n">
         <v>5.54</v>
       </c>
       <c r="BA24" s="23" t="n"/>
       <c r="BB24" s="23" t="n">
-        <v>16.988499</v>
+        <v>17.554518</v>
       </c>
       <c r="BC24" s="23" t="n"/>
       <c r="BD24" s="23" t="n">
@@ -7070,7 +7201,12 @@
       </c>
       <c r="BM24" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Extremely Overvalued</t>
+        </is>
+      </c>
+      <c r="BN24" t="inlineStr">
+        <is>
+          <t>Scored</t>
         </is>
       </c>
     </row>
@@ -7099,7 +7235,7 @@
         </is>
       </c>
       <c r="F25" s="8" t="n">
-        <v>2036360019968</v>
+        <v>2034850201600</v>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
@@ -7148,7 +7284,7 @@
         <v>1.95</v>
       </c>
       <c r="S25" s="8" t="n">
-        <v>41.2392383757963</v>
+        <v>41.20870430157542</v>
       </c>
       <c r="T25" s="8" t="n">
         <v>21.97289657631528</v>
@@ -7160,7 +7296,7 @@
         <v>0.05</v>
       </c>
       <c r="W25" s="8" t="n">
-        <v>1.730901866701827</v>
+        <v>1.732184398801846</v>
       </c>
       <c r="X25" s="8" t="n">
         <v>15.6</v>
@@ -7198,13 +7334,13 @@
         <v>2637.940388676667</v>
       </c>
       <c r="AK25" s="11" t="n">
-        <v>-181.2231857794755</v>
+        <v>-181.0146897867833</v>
       </c>
       <c r="AL25" s="15" t="n">
-        <v>3.510302394405763</v>
+        <v>3.334513164070207</v>
       </c>
       <c r="AM25" s="12" t="n">
-        <v>35103.02394405763</v>
+        <v>33345.13164070207</v>
       </c>
       <c r="AN25" s="8" t="inlineStr">
         <is>
@@ -7265,7 +7401,7 @@
       </c>
       <c r="BA25" s="23" t="n"/>
       <c r="BB25" s="23" t="n">
-        <v>37.00738</v>
+        <v>36.979946</v>
       </c>
       <c r="BC25" s="23" t="n"/>
       <c r="BD25" s="23" t="n">
@@ -7293,6 +7429,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN25" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="8" t="n">
@@ -7319,7 +7460,7 @@
         </is>
       </c>
       <c r="F26" s="8" t="n">
-        <v>246173237248</v>
+        <v>246557704192</v>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
@@ -7367,7 +7508,9 @@
       <c r="R26" s="8" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="S26" s="8" t="n"/>
+      <c r="S26" s="8" t="n">
+        <v/>
+      </c>
       <c r="T26" s="8" t="n">
         <v>9.916031751091841</v>
       </c>
@@ -7377,7 +7520,9 @@
       <c r="V26" s="8" t="n">
         <v>2.96</v>
       </c>
-      <c r="W26" s="8" t="n"/>
+      <c r="W26" s="8" t="n">
+        <v/>
+      </c>
       <c r="X26" s="8" t="n">
         <v>14</v>
       </c>
@@ -7479,7 +7624,7 @@
       <c r="AZ26" s="23" t="n"/>
       <c r="BA26" s="23" t="n"/>
       <c r="BB26" s="23" t="n">
-        <v>31.736885</v>
+        <v>31.786453</v>
       </c>
       <c r="BC26" s="23" t="n"/>
       <c r="BD26" s="23" t="n">
@@ -7502,6 +7647,11 @@
           <t>Avoid</t>
         </is>
       </c>
+      <c r="BN26" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="8" t="n">
@@ -7528,7 +7678,7 @@
         </is>
       </c>
       <c r="F27" s="8" t="n">
-        <v>1160212512768</v>
+        <v>1173429420032</v>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
@@ -7544,7 +7694,7 @@
         <v>16.66666666666667</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>12.03753444708187</v>
+        <v>12.00223309344639</v>
       </c>
       <c r="K27" s="8" t="n">
         <v>70</v>
@@ -7587,7 +7737,7 @@
         <v>0.66</v>
       </c>
       <c r="W27" s="8" t="n">
-        <v>61.7927546470487</v>
+        <v>59.76006404108044</v>
       </c>
       <c r="X27" s="8" t="n">
         <v>9.800000000000001</v>
@@ -7616,22 +7766,22 @@
         </is>
       </c>
       <c r="AH27" s="9" t="n">
-        <v>260.3949652129983</v>
+        <v>259.2193549698006</v>
       </c>
       <c r="AI27" s="10" t="n">
         <v>106</v>
       </c>
       <c r="AJ27" s="9" t="n">
-        <v>325.4937065162478</v>
+        <v>324.0241937122507</v>
       </c>
       <c r="AK27" s="11" t="n">
-        <v>68.98557545690647</v>
+        <v>68.49000723363584</v>
       </c>
       <c r="AL27" s="15" t="n">
-        <v>0.7189782118393417</v>
+        <v>0.6809702664325736</v>
       </c>
       <c r="AM27" s="12" t="n">
-        <v>7189.782118393417</v>
+        <v>6809.702664325736</v>
       </c>
       <c r="AN27" s="8" t="inlineStr">
         <is>
@@ -7679,20 +7829,20 @@
         </is>
       </c>
       <c r="AW27" s="13" t="n">
-        <v>16</v>
+        <v>15.57000032725975</v>
       </c>
       <c r="AX27" s="13" t="n">
         <v>10.6308197597</v>
       </c>
       <c r="AY27" s="23" t="n">
-        <v>20.34335665726549</v>
+        <v>20.81080242210987</v>
       </c>
       <c r="AZ27" s="23" t="n">
         <v>2.89</v>
       </c>
       <c r="BA27" s="23" t="n"/>
       <c r="BB27" s="23" t="n">
-        <v>6.309375</v>
+        <v>6.5574822</v>
       </c>
       <c r="BC27" s="23" t="n"/>
       <c r="BD27" s="23" t="n">
@@ -7720,6 +7870,11 @@
           <t>Undervalued</t>
         </is>
       </c>
+      <c r="BN27" t="inlineStr">
+        <is>
+          <t>Uncertain - Partial Data</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="8" t="n">
@@ -7746,7 +7901,7 @@
         </is>
       </c>
       <c r="F28" s="8" t="n">
-        <v>640086638592</v>
+        <v>645885919232</v>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
@@ -7795,7 +7950,7 @@
         <v>0.4</v>
       </c>
       <c r="S28" s="8" t="n">
-        <v>26.97647023015437</v>
+        <v>27.22173479517868</v>
       </c>
       <c r="T28" s="8" t="n">
         <v>16.0702848996963</v>
@@ -7807,7 +7962,7 @@
         <v>0.7</v>
       </c>
       <c r="W28" s="8" t="n">
-        <v>1.644878561676282</v>
+        <v>1.63005840315285</v>
       </c>
       <c r="X28" s="8" t="n">
         <v>35.9</v>
@@ -7836,22 +7991,22 @@
         </is>
       </c>
       <c r="AH28" s="9" t="n">
-        <v>377.5375853645027</v>
+        <v>388.5725692353753</v>
       </c>
       <c r="AI28" s="10" t="n">
         <v>1464</v>
       </c>
       <c r="AJ28" s="9" t="n">
-        <v>471.9219817056284</v>
+        <v>485.7157115442191</v>
       </c>
       <c r="AK28" s="11" t="n">
-        <v>-206.385389121779</v>
+        <v>-200.3814711616909</v>
       </c>
       <c r="AL28" s="15" t="n">
-        <v>3.636475274914664</v>
+        <v>3.454367548033276</v>
       </c>
       <c r="AM28" s="12" t="n">
-        <v>36364.75274914664</v>
+        <v>34543.67548033276</v>
       </c>
       <c r="AN28" s="8" t="inlineStr">
         <is>
@@ -7899,20 +8054,20 @@
         </is>
       </c>
       <c r="AW28" s="13" t="n">
-        <v>43.81999827253621</v>
+        <v>41.78999824132563</v>
       </c>
       <c r="AX28" s="13" t="n">
-        <v>10</v>
+        <v>11.89214301142002</v>
       </c>
       <c r="AY28" s="23" t="n">
-        <v>10.76955686229184</v>
+        <v>11.62277366700692</v>
       </c>
       <c r="AZ28" s="23" t="n">
         <v>1.06</v>
       </c>
       <c r="BA28" s="23" t="n"/>
       <c r="BB28" s="23" t="n">
-        <v>32.99635</v>
+        <v>34.91266</v>
       </c>
       <c r="BC28" s="23" t="n"/>
       <c r="BD28" s="23" t="n">
@@ -7940,6 +8095,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN28" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="8" t="n">
@@ -7966,7 +8126,7 @@
         </is>
       </c>
       <c r="F29" s="8" t="n">
-        <v>471108452352</v>
+        <v>483112910848</v>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
@@ -8015,7 +8175,7 @@
         <v>0.5</v>
       </c>
       <c r="S29" s="8" t="n">
-        <v>25.64208413289961</v>
+        <v>26.2657795218137</v>
       </c>
       <c r="T29" s="8" t="n">
         <v>35.02647805451143</v>
@@ -8027,7 +8187,7 @@
         <v>0.86</v>
       </c>
       <c r="W29" s="8" t="n">
-        <v>-3.518827208049401</v>
+        <v>-3.435270719568898</v>
       </c>
       <c r="X29" s="8" t="n">
         <v>44</v>
@@ -8065,10 +8225,10 @@
         <v/>
       </c>
       <c r="AL29" s="15" t="n">
-        <v>1.010007898123488</v>
+        <v>0.9594286342609462</v>
       </c>
       <c r="AM29" s="12" t="n">
-        <v>10100.07898123488</v>
+        <v>9594.286342609463</v>
       </c>
       <c r="AN29" s="8" t="inlineStr">
         <is>
@@ -8119,7 +8279,7 @@
         <v>33.59999716754503</v>
       </c>
       <c r="AX29" s="13" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="AY29" s="23">
         <f>IFERROR(IF(OR(T29="",T29=0,AW29="N/A",T29-AX29&lt;3),"N/A",ROUND((1-(AX29/T29))*100/(Dashboard!$B$14-AX29),1)),"N/A")</f>
@@ -8130,7 +8290,7 @@
       </c>
       <c r="BA29" s="23" t="n"/>
       <c r="BB29" s="23" t="n">
-        <v>31.068455</v>
+        <v>31.86012</v>
       </c>
       <c r="BC29" s="23" t="n"/>
       <c r="BD29" s="23" t="n">
@@ -8153,6 +8313,11 @@
           <t>Avoid</t>
         </is>
       </c>
+      <c r="BN29" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="8" t="n">
@@ -8179,7 +8344,7 @@
         </is>
       </c>
       <c r="F30" s="8" t="n">
-        <v>343745331200</v>
+        <v>349658775552</v>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
@@ -8195,7 +8360,7 @@
         <v>56.66666666666667</v>
       </c>
       <c r="J30" s="15" t="n">
-        <v>26.96942465902209</v>
+        <v>26.5698213886851</v>
       </c>
       <c r="K30" s="8" t="n">
         <v>92</v>
@@ -8238,7 +8403,7 @@
         <v>0.05</v>
       </c>
       <c r="W30" s="8" t="n">
-        <v>5.375082916147085</v>
+        <v>5.281575747474617</v>
       </c>
       <c r="X30" s="8" t="n">
         <v>26.4</v>
@@ -8276,13 +8441,13 @@
         <v>391.4289970998506</v>
       </c>
       <c r="AK30" s="11" t="n">
-        <v>-49.24801287804824</v>
+        <v>-51.81552833409818</v>
       </c>
       <c r="AL30" s="15" t="n">
-        <v>1.610830590011742</v>
+        <v>1.507490998487465</v>
       </c>
       <c r="AM30" s="12" t="n">
-        <v>16108.30590011742</v>
+        <v>15074.90998487465</v>
       </c>
       <c r="AN30" s="8" t="inlineStr">
         <is>
@@ -8341,7 +8506,7 @@
       <c r="AZ30" s="23" t="n"/>
       <c r="BA30" s="23" t="n"/>
       <c r="BB30" s="23" t="n">
-        <v>61.55954</v>
+        <v>62.618546</v>
       </c>
       <c r="BC30" s="23" t="n"/>
       <c r="BD30" s="23" t="n">
@@ -8366,7 +8531,12 @@
       </c>
       <c r="BM30" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Extremely Overvalued</t>
+        </is>
+      </c>
+      <c r="BN30" t="inlineStr">
+        <is>
+          <t>Scored</t>
         </is>
       </c>
     </row>
@@ -8395,7 +8565,7 @@
         </is>
       </c>
       <c r="F31" s="8" t="n">
-        <v>66560876544</v>
+        <v>69669879808</v>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
@@ -8444,7 +8614,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="S31" s="8" t="n">
-        <v>9.628080272458622</v>
+        <v>10.04008160612767</v>
       </c>
       <c r="T31" s="8" t="n">
         <v>14.85027274793545</v>
@@ -8456,7 +8626,7 @@
         <v>1.81</v>
       </c>
       <c r="W31" s="8" t="n">
-        <v>-1.273769076284456</v>
+        <v>-1.221499126815589</v>
       </c>
       <c r="X31" s="8" t="n">
         <v>28.5</v>
@@ -8485,22 +8655,22 @@
         </is>
       </c>
       <c r="AH31" s="9" t="n">
-        <v>44.72979551577966</v>
+        <v>33.04001064782476</v>
       </c>
       <c r="AI31" s="10" t="n">
         <v>189</v>
       </c>
       <c r="AJ31" s="9" t="n">
-        <v>55.91224439472457</v>
+        <v>41.30001330978094</v>
       </c>
       <c r="AK31" s="11" t="n">
-        <v>-228.5326890174552</v>
+        <v>-365.544644157452</v>
       </c>
       <c r="AL31" s="15" t="n">
-        <v>2.18002133336848</v>
+        <v>2.070850034360546</v>
       </c>
       <c r="AM31" s="12" t="n">
-        <v>21800.21333368481</v>
+        <v>20708.50034360546</v>
       </c>
       <c r="AN31" s="8" t="inlineStr">
         <is>
@@ -8551,15 +8721,15 @@
         <v>13.58999928754046</v>
       </c>
       <c r="AX31" s="13" t="n">
-        <v>10</v>
+        <v>21.336001</v>
       </c>
       <c r="AY31" s="23" t="n">
-        <v>4.114219602260822</v>
+        <v>3.039000243545323</v>
       </c>
       <c r="AZ31" s="23" t="n"/>
       <c r="BA31" s="23" t="n"/>
       <c r="BB31" s="23" t="n">
-        <v>13.516557</v>
+        <v>14.147903</v>
       </c>
       <c r="BC31" s="23" t="n"/>
       <c r="BD31" s="23" t="n">
@@ -8587,6 +8757,11 @@
           <t>Extremely Overvalued</t>
         </is>
       </c>
+      <c r="BN31" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="8" t="n">
@@ -8613,7 +8788,7 @@
         </is>
       </c>
       <c r="F32" s="8" t="n">
-        <v>97177214976</v>
+        <v>99996622848</v>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
@@ -8629,7 +8804,7 @@
         <v>85</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>75.44946516625131</v>
+        <v>87.45168436476672</v>
       </c>
       <c r="K32" s="8" t="n">
         <v>70</v>
@@ -8662,7 +8837,7 @@
         <v>0.3</v>
       </c>
       <c r="S32" s="8" t="n">
-        <v>10.7077203388709</v>
+        <v>10.99038758088287</v>
       </c>
       <c r="T32" s="8" t="n">
         <v>20.08202361619553</v>
@@ -8674,7 +8849,7 @@
         <v>0.5</v>
       </c>
       <c r="W32" s="8" t="n">
-        <v>9.248046492586804</v>
+        <v>9.010191387221356</v>
       </c>
       <c r="X32" s="8" t="n">
         <v>89</v>
@@ -8703,22 +8878,22 @@
         </is>
       </c>
       <c r="AH32" s="9" t="n">
-        <v>221.6136407370153</v>
+        <v>317.5164506662127</v>
       </c>
       <c r="AI32" s="10" t="n">
         <v>220</v>
       </c>
       <c r="AJ32" s="9" t="n">
-        <v>277.0170509212691</v>
+        <v>396.8955633327658</v>
       </c>
       <c r="AK32" s="11" t="n">
-        <v>27.83476708918673</v>
+        <v>48.17024451655855</v>
       </c>
       <c r="AL32" s="15" t="n">
-        <v>7.510746461126638</v>
+        <v>8.269571773046396</v>
       </c>
       <c r="AM32" s="12" t="n">
-        <v>75107.46461126639</v>
+        <v>82695.71773046395</v>
       </c>
       <c r="AN32" s="8" t="inlineStr">
         <is>
@@ -8769,17 +8944,17 @@
         <v>13.50000013506078</v>
       </c>
       <c r="AX32" s="13" t="n">
-        <v>10</v>
+        <v>21.6306065692</v>
       </c>
       <c r="AY32" s="23" t="n">
-        <v>20.51978154972364</v>
+        <v>29.39967135798265</v>
       </c>
       <c r="AZ32" s="23" t="n">
         <v>0.2</v>
       </c>
       <c r="BA32" s="23" t="n"/>
       <c r="BB32" s="23" t="n">
-        <v>14.808148</v>
+        <v>15.237779</v>
       </c>
       <c r="BC32" s="23" t="n"/>
       <c r="BD32" s="23" t="n">
@@ -8799,12 +8974,17 @@
       </c>
       <c r="BI32" s="23" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Strong Buy</t>
         </is>
       </c>
       <c r="BM32" t="inlineStr">
         <is>
           <t>Undervalued</t>
+        </is>
+      </c>
+      <c r="BN32" t="inlineStr">
+        <is>
+          <t>Scored</t>
         </is>
       </c>
     </row>
@@ -8833,7 +9013,7 @@
         </is>
       </c>
       <c r="F33" s="8" t="n">
-        <v>736226770944</v>
+        <v>739743498240</v>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
@@ -8849,7 +9029,7 @@
         <v>79.5</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>48.88575545317579</v>
+        <v>48.31977553134418</v>
       </c>
       <c r="K33" s="8" t="n">
         <v>75</v>
@@ -8882,7 +9062,7 @@
         <v>0.28</v>
       </c>
       <c r="S33" s="8" t="n">
-        <v>9.097340912335037</v>
+        <v>9.137384264258793</v>
       </c>
       <c r="T33" s="8" t="n">
         <v>21.86417857536935</v>
@@ -8894,7 +9074,7 @@
         <v>0.13</v>
       </c>
       <c r="W33" s="8" t="n">
-        <v>2.284857393098362</v>
+        <v>2.274844314295787</v>
       </c>
       <c r="X33" s="8" t="n">
         <v>60.7</v>
@@ -8923,22 +9103,22 @@
         </is>
       </c>
       <c r="AH33" s="9" t="n">
-        <v>53.90839838710311</v>
+        <v>53.78641900496129</v>
       </c>
       <c r="AI33" s="10" t="n">
         <v>88</v>
       </c>
       <c r="AJ33" s="9" t="n">
-        <v>67.38549798387888</v>
+        <v>67.2330237562016</v>
       </c>
       <c r="AK33" s="11" t="n">
-        <v>-24.27006181661479</v>
+        <v>-25.14683305797159</v>
       </c>
       <c r="AL33" s="15" t="n">
-        <v>4.866416401499921</v>
+        <v>4.569195604595232</v>
       </c>
       <c r="AM33" s="12" t="n">
-        <v>48664.16401499922</v>
+        <v>45691.95604595233</v>
       </c>
       <c r="AN33" s="8" t="inlineStr">
         <is>
@@ -8986,20 +9166,20 @@
         </is>
       </c>
       <c r="AW33" s="13" t="n">
-        <v>8.470000349526874</v>
+        <v>8.410000203903023</v>
       </c>
       <c r="AX33" s="13" t="n">
         <v>13.7094084</v>
       </c>
       <c r="AY33" s="23" t="n">
-        <v>7.955784885936112</v>
+        <v>7.994414239738597</v>
       </c>
       <c r="AZ33" s="23" t="n">
         <v>4.15</v>
       </c>
       <c r="BA33" s="23" t="n"/>
       <c r="BB33" s="23" t="n">
-        <v>9.886659</v>
+        <v>10.004756</v>
       </c>
       <c r="BC33" s="23" t="n"/>
       <c r="BD33" s="23" t="n">
@@ -9027,6 +9207,11 @@
           <t>Overvalued</t>
         </is>
       </c>
+      <c r="BN33" t="inlineStr">
+        <is>
+          <t>Scored</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="8" t="n">
@@ -9053,7 +9238,7 @@
         </is>
       </c>
       <c r="F34" s="8" t="n">
-        <v>59928293376</v>
+        <v>61246558208</v>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
@@ -9069,7 +9254,7 @@
         <v>40</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>2.445115908634934</v>
+        <v>4.084019555494167</v>
       </c>
       <c r="K34" s="8" t="n">
         <v>65</v>
@@ -9102,7 +9287,7 @@
         <v>0.38</v>
       </c>
       <c r="S34" s="8" t="n">
-        <v>16.85769966740892</v>
+        <v>17.16998109821386</v>
       </c>
       <c r="T34" s="8" t="n">
         <v>24.40495370342224</v>
@@ -9114,7 +9299,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="W34" s="8" t="n">
-        <v>2.578864848248612</v>
+        <v>2.531961383413264</v>
       </c>
       <c r="X34" s="8" t="n">
         <v>98</v>
@@ -9143,22 +9328,22 @@
         </is>
       </c>
       <c r="AH34" s="9" t="n">
-        <v>316.9243777898791</v>
+        <v>440.3269248162833</v>
       </c>
       <c r="AI34" s="10" t="n">
         <v>670</v>
       </c>
       <c r="AJ34" s="9" t="n">
-        <v>396.1554722373489</v>
+        <v>550.4086560203541</v>
       </c>
       <c r="AK34" s="11" t="n">
-        <v>-58.35954416000983</v>
+        <v>-16.48617676831926</v>
       </c>
       <c r="AL34" s="15" t="n">
-        <v>0.2434032582916017</v>
+        <v>0.3861914505364386</v>
       </c>
       <c r="AM34" s="12" t="n">
-        <v>2434.032582916017</v>
+        <v>3861.914505364386</v>
       </c>
       <c r="AN34" s="8" t="inlineStr">
         <is>
@@ -9206,20 +9391,20 @@
         </is>
       </c>
       <c r="AW34" s="13" t="n">
-        <v>42.04999965145453</v>
+        <v>41.77999663166494</v>
       </c>
       <c r="AX34" s="13" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="AY34" s="23" t="n">
-        <v>9.421057603741948</v>
+        <v>13.17397453375668</v>
       </c>
       <c r="AZ34" s="23" t="n">
         <v>0.16</v>
       </c>
       <c r="BA34" s="23" t="n"/>
       <c r="BB34" s="23" t="n">
-        <v>14.919144</v>
+        <v>15.3458605</v>
       </c>
       <c r="BC34" s="23" t="n"/>
       <c r="BD34" s="23" t="n">
@@ -9244,7 +9429,12 @@
       </c>
       <c r="BM34" t="inlineStr">
         <is>
-          <t>Extremely Overvalued</t>
+          <t>Overvalued</t>
+        </is>
+      </c>
+      <c r="BN34" t="inlineStr">
+        <is>
+          <t>Scored</t>
         </is>
       </c>
     </row>
@@ -9273,7 +9463,7 @@
         </is>
       </c>
       <c r="F35" s="8" t="n">
-        <v>99876446208</v>
+        <v>100452581376</v>
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
@@ -9289,7 +9479,7 @@
         <v>89.5</v>
       </c>
       <c r="J35" s="15" t="n">
-        <v>82.76106567344024</v>
+        <v>100</v>
       </c>
       <c r="K35" s="8" t="n">
         <v>75</v>
@@ -9322,7 +9512,7 @@
         <v>0.42</v>
       </c>
       <c r="S35" s="8" t="n">
-        <v>14.12565913611148</v>
+        <v>14.20510159851477</v>
       </c>
       <c r="T35" s="8" t="n">
         <v>24.66884209645236</v>
@@ -9334,7 +9524,7 @@
         <v>0.1</v>
       </c>
       <c r="W35" s="8" t="n">
-        <v>7.475829585599151</v>
+        <v>7.434020781440403</v>
       </c>
       <c r="X35" s="8" t="n">
         <v>36.7</v>
@@ -9363,22 +9553,22 @@
         </is>
       </c>
       <c r="AH35" s="9" t="n">
-        <v>214.2833066653625</v>
+        <v>330.6124733351869</v>
       </c>
       <c r="AI35" s="10" t="n">
         <v>262</v>
       </c>
       <c r="AJ35" s="9" t="n">
-        <v>267.8541333317031</v>
+        <v>413.2655916689836</v>
       </c>
       <c r="AK35" s="11" t="n">
-        <v>9.390981956792483</v>
+        <v>40.89757170114498</v>
       </c>
       <c r="AL35" s="15" t="n">
-        <v>8.238592278370481</v>
+        <v>9.456160659586004</v>
       </c>
       <c r="AM35" s="12" t="n">
-        <v>82385.92278370481</v>
+        <v>94561.60659586005</v>
       </c>
       <c r="AN35" s="8" t="inlineStr">
         <is>
@@ -9426,20 +9616,20 @@
         </is>
       </c>
       <c r="AW35" s="13" t="n">
-        <v>16.64999951634735</v>
+        <v>16.24997970831603</v>
       </c>
       <c r="AX35" s="13" t="n">
-        <v>10</v>
+        <v>24.70821679857</v>
       </c>
       <c r="AY35" s="23" t="n">
-        <v>16.08733533523743</v>
+        <v>25.44738864956796</v>
       </c>
       <c r="AZ35" s="23" t="n">
         <v>1.21</v>
       </c>
       <c r="BA35" s="23" t="n"/>
       <c r="BB35" s="23" t="n">
-        <v>14.576577</v>
+        <v>15.030788</v>
       </c>
       <c r="BC35" s="23" t="n"/>
       <c r="BD35" s="23" t="n">
@@ -9464,7 +9654,12 @@
       </c>
       <c r="BM35" t="inlineStr">
         <is>
-          <t>Fair Value</t>
+          <t>Undervalued</t>
+        </is>
+      </c>
+      <c r="BN35" t="inlineStr">
+        <is>
+          <t>Scored</t>
         </is>
       </c>
     </row>
@@ -9493,7 +9688,7 @@
         </is>
       </c>
       <c r="F36" s="8" t="n">
-        <v>135948935168</v>
+        <v>141948977152</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
@@ -9509,7 +9704,7 @@
         <v>89.5</v>
       </c>
       <c r="J36" s="8" t="n">
-        <v>56.15759451643354</v>
+        <v>88.07723259467328</v>
       </c>
       <c r="K36" s="8" t="n">
         <v>70</v>
@@ -9542,7 +9737,7 @@
         <v>0.75</v>
       </c>
       <c r="S36" s="8" t="n">
-        <v>15.16525565909807</v>
+        <v>15.85013254009926</v>
       </c>
       <c r="T36" s="8" t="n">
         <v>27.54079577698776</v>
@@ -9554,7 +9749,7 @@
         <v>0.13</v>
       </c>
       <c r="W36" s="8" t="n">
-        <v>5.677771639210095</v>
+        <v>5.432437758155061</v>
       </c>
       <c r="X36" s="8" t="n">
         <v>23</v>
@@ -9583,22 +9778,22 @@
         </is>
       </c>
       <c r="AH36" s="9" t="n">
-        <v>936.7003517980347</v>
+        <v>1465.447882009293</v>
       </c>
       <c r="AI36" s="10" t="n">
         <v>1400</v>
       </c>
       <c r="AJ36" s="9" t="n">
-        <v>1170.875439747543</v>
+        <v>1831.809852511616</v>
       </c>
       <c r="AK36" s="11" t="n">
-        <v>-26.17055152497911</v>
+        <v>15.79366177744596</v>
       </c>
       <c r="AL36" s="8" t="n">
-        <v>5.590304097587604</v>
+        <v>8.328724618669558</v>
       </c>
       <c r="AM36" s="12" t="n">
-        <v>55903.04097587605</v>
+        <v>83287.24618669557</v>
       </c>
       <c r="AN36" s="8" t="inlineStr">
         <is>
@@ -9649,17 +9844,17 @@
         <v>74.47000049031294</v>
       </c>
       <c r="AX36" s="13" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="AY36" s="23" t="n">
-        <v>15.72278017654819</v>
+        <v>24.59795692912067</v>
       </c>
       <c r="AZ36" s="23" t="n">
         <v>0.03</v>
       </c>
       <c r="BA36" s="23" t="n"/>
       <c r="BB36" s="23" t="n">
-        <v>19.837519</v>
+        <v>20.71304</v>
       </c>
       <c r="BC36" s="23" t="n"/>
       <c r="BD36" s="23" t="n">
@@ -9679,12 +9874,17 @@
       </c>
       <c r="BI36" s="23" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Strong Buy</t>
         </is>
       </c>
       <c r="BM36" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fair Value</t>
+        </is>
+      </c>
+      <c r="BN36" t="inlineStr">
+        <is>
+          <t>Scored</t>
         </is>
       </c>
     </row>
@@ -9713,7 +9913,7 @@
         </is>
       </c>
       <c r="F37" s="8" t="n">
-        <v>79754919936</v>
+        <v>80905232384</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -9729,7 +9929,7 @@
         <v>58</v>
       </c>
       <c r="J37" s="8" t="n">
-        <v>37.32315651577998</v>
+        <v>36.18839435014219</v>
       </c>
       <c r="K37" s="8" t="n">
         <v>35</v>
@@ -9762,7 +9962,7 @@
         <v>0.21</v>
       </c>
       <c r="S37" s="8" t="n">
-        <v>10.84749587929916</v>
+        <v>11.00837333907673</v>
       </c>
       <c r="T37" s="8" t="n">
         <v>21.70396084430917</v>
@@ -9774,7 +9974,7 @@
         <v>0.1</v>
       </c>
       <c r="W37" s="8" t="n">
-        <v>2.042240964966754</v>
+        <v>2.012395452957156</v>
       </c>
       <c r="X37" s="8" t="n">
         <v>13</v>
@@ -9812,13 +10012,13 @@
         <v>651.6784066239702</v>
       </c>
       <c r="AK37" s="11" t="n">
-        <v>-35.64973014520695</v>
+        <v>-37.60621663768589</v>
       </c>
       <c r="AL37" s="8" t="n">
-        <v>3.715397651942003</v>
+        <v>3.42203270987399</v>
       </c>
       <c r="AM37" s="12" t="n">
-        <v>37153.97651942003</v>
+        <v>34220.3270987399</v>
       </c>
       <c r="AN37" s="8" t="inlineStr">
         <is>
@@ -9879,7 +10079,7 @@
       </c>
       <c r="BA37" s="23" t="n"/>
       <c r="BB37" s="23" t="n">
-        <v>11.71016</v>
+        <v>11.879057</v>
       </c>
       <c r="BC37" s="23" t="n"/>
       <c r="BD37" s="23" t="n">
@@ -9905,6 +10105,11 @@
       <c r="BM37" t="inlineStr">
         <is>
           <t>Overvalued</t>
+        </is>
+      </c>
+      <c r="BN37" t="inlineStr">
+        <is>
+          <t>Scored</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement 4-model weighted valuation engine
</commit_message>
<xml_diff>
--- a/IOS_Master_Tracker_Filled_13.xlsx
+++ b/IOS_Master_Tracker_Filled_13.xlsx
@@ -2804,9 +2804,7 @@
       <c r="R5" s="8" t="n">
         <v>1.2</v>
       </c>
-      <c r="S5" s="8" t="n">
-        <v/>
-      </c>
+      <c r="S5" s="8" t="n"/>
       <c r="T5" s="8" t="n">
         <v>13.77443749541119</v>
       </c>
@@ -2816,9 +2814,7 @@
       <c r="V5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="W5" s="8" t="n">
-        <v/>
-      </c>
+      <c r="W5" s="8" t="n"/>
       <c r="X5" s="8" t="n">
         <v>13</v>
       </c>
@@ -2999,10 +2995,8 @@
       <c r="J6" s="8" t="n">
         <v>39.91108504814136</v>
       </c>
-      <c r="K6" s="8" t="inlineStr">
-        <is>
-          <t>±7</t>
-        </is>
+      <c r="K6" s="8" t="n">
+        <v>7</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>100</v>
@@ -3256,9 +3250,7 @@
       <c r="R7" s="8" t="n">
         <v>4.07</v>
       </c>
-      <c r="S7" s="8" t="n">
-        <v/>
-      </c>
+      <c r="S7" s="8" t="n"/>
       <c r="T7" s="8" t="n">
         <v>19.11976068675267</v>
       </c>
@@ -3268,9 +3260,7 @@
       <c r="V7" s="8" t="n">
         <v>0.08</v>
       </c>
-      <c r="W7" s="8" t="n">
-        <v/>
-      </c>
+      <c r="W7" s="8" t="n"/>
       <c r="X7" s="8" t="n">
         <v>28</v>
       </c>
@@ -4827,9 +4817,7 @@
       <c r="R14" s="8" t="n">
         <v>4.64</v>
       </c>
-      <c r="S14" s="8" t="n">
-        <v/>
-      </c>
+      <c r="S14" s="8" t="n"/>
       <c r="T14" s="8" t="n">
         <v>32.30592880341336</v>
       </c>
@@ -4839,9 +4827,7 @@
       <c r="V14" s="8" t="n">
         <v>1.5</v>
       </c>
-      <c r="W14" s="8" t="n">
-        <v/>
-      </c>
+      <c r="W14" s="8" t="n"/>
       <c r="X14" s="8" t="n">
         <v>17</v>
       </c>
@@ -5504,9 +5490,7 @@
       <c r="R17" s="8" t="n">
         <v>1.99</v>
       </c>
-      <c r="S17" s="8" t="n">
-        <v/>
-      </c>
+      <c r="S17" s="8" t="n"/>
       <c r="T17" s="8" t="n">
         <v>15.64988464815957</v>
       </c>
@@ -5516,9 +5500,7 @@
       <c r="V17" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="W17" s="8" t="n">
-        <v/>
-      </c>
+      <c r="W17" s="8" t="n"/>
       <c r="X17" s="8" t="n">
         <v>18.4</v>
       </c>
@@ -7508,9 +7490,7 @@
       <c r="R26" s="8" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="S26" s="8" t="n">
-        <v/>
-      </c>
+      <c r="S26" s="8" t="n"/>
       <c r="T26" s="8" t="n">
         <v>9.916031751091841</v>
       </c>
@@ -7520,9 +7500,7 @@
       <c r="V26" s="8" t="n">
         <v>2.96</v>
       </c>
-      <c r="W26" s="8" t="n">
-        <v/>
-      </c>
+      <c r="W26" s="8" t="n"/>
       <c r="X26" s="8" t="n">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Update tracker Excel files
</commit_message>
<xml_diff>
--- a/IOS_Master_Tracker_Filled_13.xlsx
+++ b/IOS_Master_Tracker_Filled_13.xlsx
@@ -4230,7 +4230,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>195994877952</v>
+        <v>194294661120</v>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
@@ -4279,19 +4279,19 @@
         <v>1.85</v>
       </c>
       <c r="S2" s="5" t="n">
-        <v>33.17357445625412</v>
+        <v>32.8865628548678</v>
       </c>
       <c r="T2" s="5" t="n">
-        <v>36.0316993405672</v>
+        <v>0.3603169934056724</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>41.2056152802131</v>
+        <v>0.412056152802131</v>
       </c>
       <c r="V2" s="5" t="n">
         <v>0.05</v>
       </c>
       <c r="W2" s="5" t="n">
-        <v>2.257902175505067</v>
+        <v>0.02277607613316409</v>
       </c>
       <c r="X2" s="5" t="n">
         <v>16</v>
@@ -4324,13 +4324,13 @@
         <v>521.6826793362184</v>
       </c>
       <c r="AF2" s="8" t="n">
-        <v>-51.36596081831573</v>
+        <v>-0.5005290208140002</v>
       </c>
       <c r="AG2" s="5" t="n">
-        <v>5.818282237248713</v>
+        <v>0.05805631060621214</v>
       </c>
       <c r="AH2" s="9" t="n">
-        <v>58182.82237248713</v>
+        <v>58056.31060621214</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -4381,7 +4381,7 @@
         <v>19.77999901807641</v>
       </c>
       <c r="AS2" s="8" t="n">
-        <v>13.813758</v>
+        <v>0.13813758</v>
       </c>
       <c r="AT2" s="5" t="n">
         <v>26.37425072478354</v>
@@ -4393,10 +4393,10 @@
         <v>0.133</v>
       </c>
       <c r="AW2" s="5" t="n">
-        <v>39.92164</v>
+        <v>39.575325</v>
       </c>
       <c r="AX2" s="5" t="n">
-        <v>14.824655</v>
+        <v>14.6960535</v>
       </c>
       <c r="AY2" s="5" t="n">
         <v>100</v>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>7527793164288</v>
+        <v>7489440972800</v>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
@@ -4511,19 +4511,19 @@
         <v>1.66</v>
       </c>
       <c r="S3" s="5" t="n">
-        <v>11.32307774206678</v>
+        <v>11.26585445495509</v>
       </c>
       <c r="T3" s="5" t="n">
-        <v>45.3640369475838</v>
+        <v>0.4536403694758384</v>
       </c>
       <c r="U3" s="5" t="n">
-        <v>55.1812149055641</v>
+        <v>0.5518121490556407</v>
       </c>
       <c r="V3" s="5" t="n">
         <v>0.11</v>
       </c>
       <c r="W3" s="5" t="n">
-        <v>6.318130967737829</v>
+        <v>0.06350223005125825</v>
       </c>
       <c r="X3" s="5" t="n">
         <v>6</v>
@@ -4556,13 +4556,13 @@
         <v>4190.507996530057</v>
       </c>
       <c r="AF3" s="8" t="n">
-        <v>50.34969503165637</v>
+        <v>0.5060264765718</v>
       </c>
       <c r="AG3" s="5" t="n">
-        <v>12.19409725391108</v>
+        <v>0.1216758261060545</v>
       </c>
       <c r="AH3" s="9" t="n">
-        <v>121940.9725391108</v>
+        <v>121675.8261060545</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
@@ -4613,7 +4613,7 @@
         <v>135.4699993788408</v>
       </c>
       <c r="AS3" s="8" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT3" s="5" t="n">
         <v>30.93310693533665</v>
@@ -4625,10 +4625,10 @@
         <v>0.241</v>
       </c>
       <c r="AW3" s="5" t="n">
-        <v>15.358382</v>
+        <v>15.280136</v>
       </c>
       <c r="AX3" s="5" t="n">
-        <v>7.0195684</v>
+        <v>6.9838057</v>
       </c>
       <c r="AY3" s="5" t="n">
         <v>100</v>
@@ -4694,7 +4694,7 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>1144641814528</v>
+        <v>1146333560832</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
@@ -4743,19 +4743,19 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="S4" s="5" t="n">
-        <v>7.967674470988738</v>
+        <v>7.979197419562253</v>
       </c>
       <c r="T4" s="5" t="n">
-        <v>23.6874355105433</v>
+        <v>0.2368743551054329</v>
       </c>
       <c r="U4" s="5" t="n">
-        <v>57.0964225532102</v>
+        <v>0.5709642255321019</v>
       </c>
       <c r="V4" s="5" t="n">
         <v>0.29</v>
       </c>
       <c r="W4" s="5" t="n">
-        <v>4.513380396789722</v>
+        <v>0.04506862516924084</v>
       </c>
       <c r="X4" s="5" t="n">
         <v>23</v>
@@ -4788,13 +4788,13 @@
         <v>3231.91809180553</v>
       </c>
       <c r="AF4" s="8" t="n">
-        <v>22.53825966853619</v>
+        <v>0.2242687070700506</v>
       </c>
       <c r="AG4" s="5" t="n">
-        <v>12.19409725391108</v>
+        <v>0.1216758261060545</v>
       </c>
       <c r="AH4" s="9" t="n">
-        <v>121940.9725391108</v>
+        <v>121675.8261060545</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
@@ -4842,10 +4842,10 @@
         </is>
       </c>
       <c r="AR4" s="8" t="n">
-        <v>116.5646599790011</v>
+        <v>116.5599893180076</v>
       </c>
       <c r="AS4" s="8" t="n">
-        <v>24.1328883</v>
+        <v>0.241328883</v>
       </c>
       <c r="AT4" s="5" t="n">
         <v>27.72750593518814</v>
@@ -4857,10 +4857,10 @@
         <v>0.18</v>
       </c>
       <c r="AW4" s="5" t="n">
-        <v>21.47735</v>
+        <v>21.509096</v>
       </c>
       <c r="AX4" s="5" t="n">
-        <v>5.095596</v>
+        <v>5.1031275</v>
       </c>
       <c r="AY4" s="5" t="n">
         <v>100</v>
@@ -4936,7 +4936,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>77386178560</v>
+        <v>77266386944</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
@@ -4985,19 +4985,19 @@
         <v>1.2</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v/>
+        <v>17.67514266764074</v>
       </c>
       <c r="T5" s="5" t="n">
-        <v>13.7744374954112</v>
+        <v>0.1377443749541119</v>
       </c>
       <c r="U5" s="5" t="n">
-        <v>12.9445748330024</v>
+        <v>0.1294457483300235</v>
       </c>
       <c r="V5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="W5" s="5" t="n">
-        <v/>
+        <v>0.008205120554582066</v>
       </c>
       <c r="X5" s="5" t="n">
         <v>13</v>
@@ -5030,13 +5030,13 @@
         <v>401.2047387412738</v>
       </c>
       <c r="AF5" s="8" t="n">
-        <v>-173.7505054017481</v>
+        <v>-1.733267815929681</v>
       </c>
       <c r="AG5" s="5" t="n">
-        <v>2.660738412210071</v>
+        <v>0.02654952946631083</v>
       </c>
       <c r="AH5" s="9" t="n">
-        <v>26607.38412210071</v>
+        <v>26549.52946631083</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
@@ -5087,7 +5087,7 @@
         <v>58.55999984644195</v>
       </c>
       <c r="AS5" s="8" t="n">
-        <v>13.044297</v>
+        <v>0.13044297</v>
       </c>
       <c r="AT5" s="5" t="n">
         <v>6.851173817303173</v>
@@ -5099,10 +5099,10 @@
         <v>0.509</v>
       </c>
       <c r="AW5" s="5" t="n">
-        <v>18.755123</v>
+        <v>18.726091</v>
       </c>
       <c r="AX5" s="5" t="n">
-        <v>2.581854</v>
+        <v>2.5778575</v>
       </c>
       <c r="AY5" s="5" t="n">
         <v>100</v>
@@ -5168,7 +5168,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>776327659520</v>
+        <v>772874960896</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
@@ -5217,19 +5217,19 @@
         <v>1.04</v>
       </c>
       <c r="S6" s="5" t="n">
-        <v>32.19875625634015</v>
+        <v>32.05444241199451</v>
       </c>
       <c r="T6" s="5" t="n">
-        <v>23.796306514984</v>
+        <v>0.2379630651498401</v>
       </c>
       <c r="U6" s="5" t="n">
-        <v>28.3058622706657</v>
+        <v>0.2830586227066565</v>
       </c>
       <c r="V6" s="5" t="n">
         <v>0.06</v>
       </c>
       <c r="W6" s="5" t="n">
-        <v>2.02316213632288</v>
+        <v>0.02032270711723274</v>
       </c>
       <c r="X6" s="5" t="n">
         <v>19.6</v>
@@ -5262,13 +5262,13 @@
         <v>2812.70299797622</v>
       </c>
       <c r="AF6" s="8" t="n">
-        <v>-76.66635985297201</v>
+        <v>-0.7588063878622935</v>
       </c>
       <c r="AG6" s="10" t="n">
-        <v>5.07725973056198</v>
+        <v>0.05066219821012079</v>
       </c>
       <c r="AH6" s="9" t="n">
-        <v>50772.59730561981</v>
+        <v>50662.19821012079</v>
       </c>
       <c r="AI6" s="5" t="inlineStr">
         <is>
@@ -5319,7 +5319,7 @@
         <v>120.2600022652666</v>
       </c>
       <c r="AS6" s="8" t="n">
-        <v>18.14655820438</v>
+        <v>0.1814655820438004</v>
       </c>
       <c r="AT6" s="5" t="n">
         <v>23.38851653065208</v>
@@ -5331,10 +5331,10 @@
         <v>0.121</v>
       </c>
       <c r="AW6" s="5" t="n">
-        <v>41.31964</v>
+        <v>41.13587</v>
       </c>
       <c r="AX6" s="5" t="n">
-        <v>9.918542</v>
+        <v>9.874428999999999</v>
       </c>
       <c r="AY6" s="5" t="n">
         <v>100</v>
@@ -5400,7 +5400,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>251128152064</v>
+        <v>252858679296</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
@@ -5449,19 +5449,19 @@
         <v>4.07</v>
       </c>
       <c r="S7" s="5" t="n">
-        <v/>
+        <v>36.61228221886392</v>
       </c>
       <c r="T7" s="5" t="n">
-        <v>19.1197606867527</v>
+        <v>0.1911976068675267</v>
       </c>
       <c r="U7" s="5" t="n">
-        <v>25.4768608936117</v>
+        <v>0.2547686089361172</v>
       </c>
       <c r="V7" s="5" t="n">
         <v>0.08</v>
       </c>
       <c r="W7" s="5" t="n">
-        <v/>
+        <v>0.0001667282056983589</v>
       </c>
       <c r="X7" s="5" t="n">
         <v>28</v>
@@ -5494,13 +5494,13 @@
         <v>178.6734617775119</v>
       </c>
       <c r="AF7" s="8" t="n">
-        <v>-1142.657962694408</v>
+        <v>-11.51221069855252</v>
       </c>
       <c r="AG7" s="10" t="n">
-        <v>3.411125288679415</v>
+        <v>0.03403708194292118</v>
       </c>
       <c r="AH7" s="9" t="n">
-        <v>34111.25288679415</v>
+        <v>34037.08194292118</v>
       </c>
       <c r="AI7" s="5" t="inlineStr">
         <is>
@@ -5551,7 +5551,7 @@
         <v>43.90999880094436</v>
       </c>
       <c r="AS7" s="8" t="n">
-        <v>17.2376802</v>
+        <v>0.172376802</v>
       </c>
       <c r="AT7" s="5" t="n">
         <v>4.069083620530901</v>
@@ -5563,10 +5563,10 @@
         <v>1.45</v>
       </c>
       <c r="AW7" s="5" t="n">
-        <v>50.564793</v>
+        <v>50.913235</v>
       </c>
       <c r="AX7" s="5" t="n">
-        <v>9.754844</v>
+        <v>9.822063999999999</v>
       </c>
       <c r="AY7" s="5" t="n">
         <v>100</v>
@@ -5632,7 +5632,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>1569645002752</v>
+        <v>1562160660480</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
@@ -5681,19 +5681,19 @@
         <v>2.05</v>
       </c>
       <c r="S8" s="5" t="n">
-        <v>65.30807280872995</v>
+        <v>64.99575022346485</v>
       </c>
       <c r="T8" s="5" t="n">
-        <v>27.8667305396004</v>
+        <v>0.2786673053960043</v>
       </c>
       <c r="U8" s="5" t="n">
-        <v>27.0330790985627</v>
+        <v>0.270330790985627</v>
       </c>
       <c r="V8" s="5" t="n">
         <v>0.003</v>
       </c>
       <c r="W8" s="5" t="n">
-        <v>0.9473102391633295</v>
+        <v>0.009518623272910354</v>
       </c>
       <c r="X8" s="5" t="n">
         <v>13</v>
@@ -5726,13 +5726,13 @@
         <v>1726.318101537442</v>
       </c>
       <c r="AF8" s="8" t="n">
-        <v>-228.0102314258904</v>
+        <v>-2.264462091303498</v>
       </c>
       <c r="AG8" s="10" t="n">
-        <v>5.449022684609782</v>
+        <v>0.0543717441984378</v>
       </c>
       <c r="AH8" s="9" t="n">
-        <v>54490.22684609782</v>
+        <v>54371.7441984378</v>
       </c>
       <c r="AI8" s="5" t="inlineStr">
         <is>
@@ -5783,7 +5783,7 @@
         <v>85.91000773076281</v>
       </c>
       <c r="AS8" s="8" t="n">
-        <v>10.9602055</v>
+        <v>0.109602055</v>
       </c>
       <c r="AT8" s="5" t="n">
         <v>20.09449542006102</v>
@@ -5795,10 +5795,10 @@
         <v>0.572</v>
       </c>
       <c r="AW8" s="5" t="n">
-        <v>65.911995</v>
+        <v>65.59772</v>
       </c>
       <c r="AX8" s="5" t="n">
-        <v>18.519972</v>
+        <v>18.431665</v>
       </c>
       <c r="AY8" s="5" t="n">
         <v>100</v>
@@ -5874,7 +5874,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>213748400128</v>
+        <v>214548152320</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
@@ -5923,19 +5923,19 @@
         <v>2.49</v>
       </c>
       <c r="S9" s="5" t="n">
-        <v>159.7169136134997</v>
+        <v>160.3041851065861</v>
       </c>
       <c r="T9" s="5" t="n">
-        <v>11.4310097290621</v>
+        <v>0.1143100972906209</v>
       </c>
       <c r="U9" s="5" t="n">
-        <v>13.3959153480375</v>
+        <v>0.1339591534803745</v>
       </c>
       <c r="V9" s="5" t="n">
         <v>0.3</v>
       </c>
       <c r="W9" s="5" t="n">
-        <v>0.2910290099038979</v>
+        <v>0.002899628303711297</v>
       </c>
       <c r="X9" s="5" t="n">
         <v>29.6</v>
@@ -5968,7 +5968,7 @@
         <v>615.7168663403008</v>
       </c>
       <c r="AF9" s="8" t="n">
-        <v>-1028.60315834833</v>
+        <v>-10.32825878468787</v>
       </c>
       <c r="AG9" s="10" t="n">
         <v>0.672326191827808</v>
@@ -6025,7 +6025,7 @@
         <v>31.21999977716046</v>
       </c>
       <c r="AS9" s="8" t="n">
-        <v>12.121</v>
+        <v>0.12121</v>
       </c>
       <c r="AT9" s="5" t="n">
         <v>19.7218727207015</v>
@@ -6035,10 +6035,10 @@
         <v>1.099</v>
       </c>
       <c r="AW9" s="5" t="n">
-        <v>222.58168</v>
+        <v>223.41449</v>
       </c>
       <c r="AX9" s="5" t="n">
-        <v>25.978542</v>
+        <v>26.075743</v>
       </c>
       <c r="AY9" s="5" t="n">
         <v>75</v>
@@ -6104,7 +6104,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>443874607104</v>
+        <v>439346692096</v>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
@@ -6153,19 +6153,19 @@
         <v>1.13</v>
       </c>
       <c r="S10" s="5" t="n">
-        <v>38.92529576968217</v>
+        <v>38.5637942481218</v>
       </c>
       <c r="T10" s="5" t="n">
-        <v>10.224468143237</v>
+        <v>0.1022446814323704</v>
       </c>
       <c r="U10" s="5" t="n">
-        <v>11.3635373912665</v>
+        <v>0.1136353739126648</v>
       </c>
       <c r="V10" s="5" t="n">
         <v>0.1</v>
       </c>
       <c r="W10" s="5" t="n">
-        <v>2.47524870714209</v>
+        <v>0.024984519782755</v>
       </c>
       <c r="X10" s="5" t="n">
         <v>-0.1</v>
@@ -6198,7 +6198,7 @@
         <v>814.2752106976557</v>
       </c>
       <c r="AF10" s="8" t="n">
-        <v>-55.30375767137924</v>
+        <v>-0.5371952670984138</v>
       </c>
       <c r="AG10" s="10" t="n">
         <v>0.539014569111855</v>
@@ -6255,7 +6255,7 @@
         <v>25.53000088020563</v>
       </c>
       <c r="AS10" s="8" t="n">
-        <v>10.48834958224</v>
+        <v>0.1048834958223998</v>
       </c>
       <c r="AT10" s="5" t="n">
         <v>31.89483786516473</v>
@@ -6267,10 +6267,10 @@
         <v>0.572</v>
       </c>
       <c r="AW10" s="5" t="n">
-        <v>49.53388</v>
+        <v>49.02859</v>
       </c>
       <c r="AX10" s="5" t="n">
-        <v>7.3316097</v>
+        <v>7.2568207</v>
       </c>
       <c r="AY10" s="5" t="n">
         <v>100</v>
@@ -6336,7 +6336,7 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>250824327168</v>
+        <v>250554908672</v>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
@@ -6385,19 +6385,19 @@
         <v>1.66</v>
       </c>
       <c r="S11" s="5" t="n">
-        <v>52.42174917924767</v>
+        <v>52.36594102514654</v>
       </c>
       <c r="T11" s="5" t="n">
-        <v>19.4187069869082</v>
+        <v>0.1941870698690816</v>
       </c>
       <c r="U11" s="5" t="n">
-        <v>21.7464600502437</v>
+        <v>0.2174646005024371</v>
       </c>
       <c r="V11" s="5" t="n">
         <v>0.4</v>
       </c>
       <c r="W11" s="5" t="n">
-        <v>-0.1993584035557694</v>
+        <v>-0.001995708665477292</v>
       </c>
       <c r="X11" s="5" t="n">
         <v>37</v>
@@ -6430,7 +6430,7 @@
         <v>1862.084374558736</v>
       </c>
       <c r="AF11" s="8" t="n">
-        <v>-949.8987192582408</v>
+        <v>-9.487709508130019</v>
       </c>
       <c r="AG11" s="10" t="n">
         <v>1.14589975174742</v>
@@ -6487,7 +6487,7 @@
         <v>293.1300189519428</v>
       </c>
       <c r="AS11" s="8" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="AT11" s="5" t="n">
         <v>6.352418294131398</v>
@@ -6499,10 +6499,10 @@
         <v>-0.321</v>
       </c>
       <c r="AW11" s="5" t="n">
-        <v>66.69395400000001</v>
+        <v>66.622314</v>
       </c>
       <c r="AX11" s="5" t="n">
-        <v>13.390219</v>
+        <v>13.375835</v>
       </c>
       <c r="AY11" s="5" t="n">
         <v>50</v>
@@ -6568,7 +6568,7 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>116553334784</v>
+        <v>109058367488</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -6617,19 +6617,19 @@
         <v>1.85</v>
       </c>
       <c r="S12" s="5" t="n">
-        <v>27.39882442482</v>
+        <v>25.65243784234686</v>
       </c>
       <c r="T12" s="5" t="n">
-        <v>14.7951063174649</v>
+        <v>0.1479510631746486</v>
       </c>
       <c r="U12" s="5" t="n">
-        <v>16.7132687394853</v>
+        <v>0.1671326873948533</v>
       </c>
       <c r="V12" s="5" t="n">
         <v>0.12</v>
       </c>
       <c r="W12" s="5" t="n">
-        <v>1.655787752993123</v>
+        <v>0.01768511757355665</v>
       </c>
       <c r="X12" s="5" t="n">
         <v>17.5</v>
@@ -6662,13 +6662,13 @@
         <v>233.8382459449688</v>
       </c>
       <c r="AF12" s="8" t="n">
-        <v>-122.11935344496</v>
+        <v>-1.078359756916644</v>
       </c>
       <c r="AG12" s="10" t="n">
-        <v>2.606247512647069</v>
+        <v>0.02600580531178485</v>
       </c>
       <c r="AH12" s="9" t="n">
-        <v>26062.47512647069</v>
+        <v>26005.80531178485</v>
       </c>
       <c r="AI12" s="5" t="inlineStr">
         <is>
@@ -6719,7 +6719,7 @@
         <v>15.1899992834906</v>
       </c>
       <c r="AS12" s="8" t="n">
-        <v>13.76500855851</v>
+        <v>0.1376500855851</v>
       </c>
       <c r="AT12" s="5" t="n">
         <v>15.39422290618623</v>
@@ -6731,10 +6731,10 @@
         <v>0.489</v>
       </c>
       <c r="AW12" s="5" t="n">
-        <v>34.19355</v>
+        <v>31.994734</v>
       </c>
       <c r="AX12" s="5" t="n">
-        <v>5.054693</v>
+        <v>4.729651</v>
       </c>
       <c r="AY12" s="5" t="n">
         <v>100</v>
@@ -6800,7 +6800,7 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>9477074976768</v>
+        <v>9469690904576</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
@@ -6816,7 +6816,7 @@
         <v>23.33333333333334</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>14.13939286769403</v>
+        <v>14.15019299013081</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>75</v>
@@ -6850,7 +6850,7 @@
       </c>
       <c r="S13" s="5" t="n"/>
       <c r="T13" s="5" t="n">
-        <v>13.546738870871</v>
+        <v>0.1354673887087101</v>
       </c>
       <c r="U13" s="5" t="n">
         <v>13.76</v>
@@ -6859,7 +6859,7 @@
         <v>1.33</v>
       </c>
       <c r="W13" s="5" t="n">
-        <v>2.897374000206035</v>
+        <v>0.02899460210105789</v>
       </c>
       <c r="X13" s="5" t="n">
         <v>5.2</v>
@@ -6892,13 +6892,13 @@
         <v>1037.025280551953</v>
       </c>
       <c r="AF13" s="8" t="n">
-        <v>0.9956633406716405</v>
+        <v>0.01072807072362944</v>
       </c>
       <c r="AG13" s="10" t="n">
-        <v>1.034502790439506</v>
+        <v>0.01033041852980561</v>
       </c>
       <c r="AH13" s="9" t="n">
-        <v>10345.02790439506</v>
+        <v>10330.41852980561</v>
       </c>
       <c r="AI13" s="5" t="inlineStr">
         <is>
@@ -6949,7 +6949,7 @@
         <v>91.58000892340907</v>
       </c>
       <c r="AS13" s="8" t="n">
-        <v>12.7778112</v>
+        <v>0.127778112</v>
       </c>
       <c r="AT13" s="5" t="n">
         <v>11.32370911281888</v>
@@ -6961,10 +6961,10 @@
         <v>0.362</v>
       </c>
       <c r="AW13" s="5" t="n">
-        <v>11.210962</v>
+        <v>11.202228</v>
       </c>
       <c r="AX13" s="5" t="n">
-        <v>1.5897644</v>
+        <v>1.5885257</v>
       </c>
       <c r="AY13" s="5" t="n">
         <v>60</v>
@@ -7040,7 +7040,7 @@
         </is>
       </c>
       <c r="F14" s="5" t="n">
-        <v>4059207827456</v>
+        <v>4074642341888</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
@@ -7089,19 +7089,19 @@
         <v>4.64</v>
       </c>
       <c r="S14" s="5" t="n">
-        <v/>
+        <v>57.8499118597829</v>
       </c>
       <c r="T14" s="5" t="n">
-        <v>32.3059288034134</v>
+        <v>0.3230592880341336</v>
       </c>
       <c r="U14" s="5" t="n">
-        <v>36.3732665639445</v>
+        <v>0.3637326656394453</v>
       </c>
       <c r="V14" s="5" t="n">
         <v>1.5</v>
       </c>
       <c r="W14" s="5" t="n">
-        <v/>
+        <v>0.01072773213535367</v>
       </c>
       <c r="X14" s="5" t="n">
         <v>17</v>
@@ -7134,7 +7134,7 @@
         <v>1549.492432635347</v>
       </c>
       <c r="AF14" s="8" t="n">
-        <v>-195.3289673197731</v>
+        <v>-1.964519156887693</v>
       </c>
       <c r="AG14" s="10">
         <f>IF(H14="Fail","Not Eligible (Failed Gate)",IF(J14="","Pending Score",IF(J14&gt;=90,"10%",IF(J14&gt;=80,"7.5%",IF(J14&gt;=70,"5%","Watchlist only")))))</f>
@@ -7193,7 +7193,7 @@
         <v>56.95000083382139</v>
       </c>
       <c r="AS14" s="8" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT14" s="5" t="n">
         <v>27.20794438341258</v>
@@ -7205,10 +7205,10 @@
         <v>0.219</v>
       </c>
       <c r="AW14" s="5" t="n">
-        <v>80.35294</v>
+        <v>80.65846999999999</v>
       </c>
       <c r="AX14" s="5" t="n">
-        <v>25.871944</v>
+        <v>25.970318</v>
       </c>
       <c r="AY14" s="5" t="n">
         <v>100</v>
@@ -7274,7 +7274,7 @@
         </is>
       </c>
       <c r="F15" s="5" t="n">
-        <v>1287188381696</v>
+        <v>1282847801344</v>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
@@ -7323,19 +7323,19 @@
         <v>2.66</v>
       </c>
       <c r="S15" s="5" t="n">
-        <v>17.09830102865496</v>
+        <v>17.03954846903721</v>
       </c>
       <c r="T15" s="5" t="n">
-        <v>15.9952787844532</v>
+        <v>0.1599527878445324</v>
       </c>
       <c r="U15" s="5" t="n">
-        <v>21.1858258368486</v>
+        <v>0.2118582583684858</v>
       </c>
       <c r="V15" s="5" t="n">
         <v>0.1</v>
       </c>
       <c r="W15" s="5" t="n">
-        <v>4.335241188291512</v>
+        <v>0.04350189149901837</v>
       </c>
       <c r="X15" s="5" t="n">
         <v>8.460000000000001</v>
@@ -7368,7 +7368,7 @@
         <v>900.641159790913</v>
       </c>
       <c r="AF15" s="8" t="n">
-        <v>-61.34061653781649</v>
+        <v>-0.607965596793516</v>
       </c>
       <c r="AG15" s="10" t="n">
         <v>2.1360059695849</v>
@@ -7425,7 +7425,7 @@
         <v>54.06000053647045</v>
       </c>
       <c r="AS15" s="8" t="n">
-        <v>5</v>
+        <v>0.05</v>
       </c>
       <c r="AT15" s="5" t="n">
         <v>16.66002885295806</v>
@@ -7437,10 +7437,10 @@
         <v>0.173</v>
       </c>
       <c r="AW15" s="5" t="n">
-        <v>26.879393</v>
+        <v>26.788752</v>
       </c>
       <c r="AX15" s="5" t="n">
-        <v>4.3452907</v>
+        <v>4.330638</v>
       </c>
       <c r="AY15" s="5" t="n">
         <v>100</v>
@@ -7516,7 +7516,7 @@
         </is>
       </c>
       <c r="F16" s="5" t="n">
-        <v>5409091878912</v>
+        <v>5400149622784</v>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
@@ -7565,19 +7565,19 @@
         <v>2.5</v>
       </c>
       <c r="S16" s="5" t="n">
-        <v>24.7595690778288</v>
+        <v>24.72653594949792</v>
       </c>
       <c r="T16" s="5" t="n">
-        <v>12.5137574392872</v>
+        <v>0.1251375743928715</v>
       </c>
       <c r="U16" s="5" t="n">
-        <v>13.6683898304272</v>
+        <v>0.1366838983042717</v>
       </c>
       <c r="V16" s="5" t="n">
         <v>1.12</v>
       </c>
       <c r="W16" s="5" t="n">
-        <v>1.780183432626119</v>
+        <v>0.01782561647993712</v>
       </c>
       <c r="X16" s="5" t="n">
         <v>12</v>
@@ -7610,7 +7610,7 @@
         <v>2359.753407960584</v>
       </c>
       <c r="AF16" s="8" t="n">
-        <v>-66.61910463763488</v>
+        <v>-0.6634365212729741</v>
       </c>
       <c r="AG16" s="10" t="n">
         <v>0.0283377540664614</v>
@@ -7667,7 +7667,7 @@
         <v>116.5800020850261</v>
       </c>
       <c r="AS16" s="8" t="n">
-        <v>12.0206624909</v>
+        <v>0.120206624909</v>
       </c>
       <c r="AT16" s="5" t="n">
         <v>20.24149432115787</v>
@@ -7679,10 +7679,10 @@
         <v>0.46</v>
       </c>
       <c r="AW16" s="5" t="n">
-        <v>33.726196</v>
+        <v>33.67044</v>
       </c>
       <c r="AX16" s="5" t="n">
-        <v>4.94896</v>
+        <v>4.9407783</v>
       </c>
       <c r="AY16" s="5" t="n">
         <v>100</v>
@@ -7758,7 +7758,7 @@
         </is>
       </c>
       <c r="F17" s="5" t="n">
-        <v>115824861184</v>
+        <v>117421662208</v>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
@@ -7807,19 +7807,19 @@
         <v>1.99</v>
       </c>
       <c r="S17" s="5" t="n">
-        <v/>
+        <v>85.04757121346577</v>
       </c>
       <c r="T17" s="5" t="n">
-        <v>15.6498846481596</v>
+        <v>0.1564988464815957</v>
       </c>
       <c r="U17" s="5" t="n">
-        <v>18.1829538386265</v>
+        <v>0.1818295383862648</v>
       </c>
       <c r="V17" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="W17" s="5" t="n">
-        <v/>
+        <v>0.0002983035685383026</v>
       </c>
       <c r="X17" s="5" t="n">
         <v>18.4</v>
@@ -7852,7 +7852,7 @@
         <v>64.8379065093409</v>
       </c>
       <c r="AF17" s="8" t="n">
-        <v>-2573.744562912821</v>
+        <v>-26.10605716035581</v>
       </c>
       <c r="AG17" s="10" t="n">
         <v>0.805381150830505</v>
@@ -7909,7 +7909,7 @@
         <v>16.7999984462429</v>
       </c>
       <c r="AS17" s="8" t="n">
-        <v>16.943</v>
+        <v>0.16943</v>
       </c>
       <c r="AT17" s="5" t="n">
         <v>3.85939919698458</v>
@@ -7917,10 +7917,10 @@
       <c r="AU17" s="5" t="n"/>
       <c r="AV17" s="5" t="n"/>
       <c r="AW17" s="5" t="n">
-        <v>103.19048</v>
+        <v>104.6131</v>
       </c>
       <c r="AX17" s="5" t="n">
-        <v>16.0468</v>
+        <v>16.268026</v>
       </c>
       <c r="AY17" s="5" t="n">
         <v>75</v>
@@ -7986,7 +7986,7 @@
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>1450555867136</v>
+        <v>1448350842880</v>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
@@ -8035,19 +8035,19 @@
         <v>3.84</v>
       </c>
       <c r="S18" s="5" t="n">
-        <v>100.4000793739405</v>
+        <v>100.2475068245193</v>
       </c>
       <c r="T18" s="5" t="n">
-        <v>14.7137498856463</v>
+        <v>0.1471374988564633</v>
       </c>
       <c r="U18" s="5" t="n">
-        <v>17.0673005953119</v>
+        <v>0.170673005953119</v>
       </c>
       <c r="V18" s="5" t="n">
         <v>0.1</v>
       </c>
       <c r="W18" s="5" t="n">
-        <v>-0.051901704820861</v>
+        <v>-0.0005198069706390686</v>
       </c>
       <c r="X18" s="5" t="n">
         <v>25</v>
@@ -8080,7 +8080,7 @@
         <v>80.26805595178079</v>
       </c>
       <c r="AF18" s="8" t="n">
-        <v>-1047.405389453146</v>
+        <v>-10.45661233595128</v>
       </c>
       <c r="AG18" s="10" t="n">
         <v>0.741456322052803</v>
@@ -8137,7 +8137,7 @@
         <v>7.73999982817047</v>
       </c>
       <c r="AS18" s="8" t="n">
-        <v>16.2591032</v>
+        <v>0.162591032</v>
       </c>
       <c r="AT18" s="5" t="n">
         <v>10.3705498645712</v>
@@ -8149,10 +8149,10 @@
         <v>0.407</v>
       </c>
       <c r="AW18" s="5" t="n">
-        <v>118.99225</v>
+        <v>118.81137</v>
       </c>
       <c r="AX18" s="5" t="n">
-        <v>18.198343</v>
+        <v>18.170681</v>
       </c>
       <c r="AY18" s="5" t="n">
         <v>50</v>
@@ -8218,7 +8218,7 @@
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>97688657920</v>
+        <v>98621145088</v>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
@@ -8266,16 +8266,16 @@
       <c r="R19" s="5" t="n"/>
       <c r="S19" s="5" t="n"/>
       <c r="T19" s="5" t="n">
-        <v>-31.0109284956344</v>
+        <v>-0.310109284956344</v>
       </c>
       <c r="U19" s="5" t="n">
-        <v>-29.3683699950399</v>
+        <v>-0.2936836999503991</v>
       </c>
       <c r="V19" s="5" t="n">
         <v>0.9</v>
       </c>
       <c r="W19" s="5" t="n">
-        <v>-5.4084058722088</v>
+        <v>-0.05372218423245244</v>
       </c>
       <c r="X19" s="5" t="n">
         <v>-88</v>
@@ -8365,7 +8365,7 @@
         <v/>
       </c>
       <c r="AS19" s="8" t="n">
-        <v>5</v>
+        <v>0.05</v>
       </c>
       <c r="AT19" s="5">
         <f>IFERROR(IF(OR(T19="",T19=0,AR19="N/A",T19-AS19&lt;3),"N/A",ROUND((1-(AS19/T19))*100/(Dashboard!$B$14-AS19),1)),"N/A")</f>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="AW19" s="5" t="n"/>
       <c r="AX19" s="5" t="n">
-        <v>3.335456</v>
+        <v>3.3672943</v>
       </c>
       <c r="AY19" s="5" t="n">
         <v>0</v>
@@ -8451,7 +8451,7 @@
         </is>
       </c>
       <c r="F20" s="5" t="n">
-        <v>262528548864</v>
+        <v>261998821376</v>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
@@ -8500,19 +8500,19 @@
         <v>0.57</v>
       </c>
       <c r="S20" s="5" t="n">
-        <v>33.43669486734773</v>
+        <v>33.39636337844155</v>
       </c>
       <c r="T20" s="5" t="n">
-        <v>9.85965288109011</v>
+        <v>0.09859652881090114</v>
       </c>
       <c r="U20" s="5" t="n">
-        <v>5.18730734217609</v>
+        <v>0.05187307342176093</v>
       </c>
       <c r="V20" s="5" t="n">
         <v>0.65</v>
       </c>
       <c r="W20" s="5" t="n">
-        <v>-9.273454529830218</v>
+        <v>-0.09284653720120896</v>
       </c>
       <c r="X20" s="5" t="n">
         <v>42.3</v>
@@ -8545,7 +8545,7 @@
         <v>67.29377072908061</v>
       </c>
       <c r="AF20" s="8" t="n">
-        <v>-452.3542461254473</v>
+        <v>-4.512397298903274</v>
       </c>
       <c r="AG20" s="10">
         <f>IF(H20="Fail","Not Eligible (Failed Gate)",IF(J20="","Pending Score",IF(J20&gt;=90,"10%",IF(J20&gt;=80,"7.5%",IF(J20&gt;=70,"5%","Watchlist only")))))</f>
@@ -8604,7 +8604,7 @@
         <v>8.14999980364135</v>
       </c>
       <c r="AS20" s="8" t="n">
-        <v>9.896105979188</v>
+        <v>0.09896105979188</v>
       </c>
       <c r="AT20" s="5" t="n">
         <v>8.25690438393627</v>
@@ -8614,10 +8614,10 @@
       </c>
       <c r="AV20" s="5" t="n"/>
       <c r="AW20" s="5" t="n">
-        <v>45.607365</v>
+        <v>45.515343</v>
       </c>
       <c r="AX20" s="5" t="n">
-        <v>4.448248</v>
+        <v>4.4392724</v>
       </c>
       <c r="AY20" s="5" t="n">
         <v>50</v>
@@ -8693,7 +8693,7 @@
         </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>13706356736</v>
+        <v>13649467392</v>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
@@ -8742,19 +8742,19 @@
         <v>5.08</v>
       </c>
       <c r="S21" s="5" t="n">
-        <v>22.83138789393477</v>
+        <v>22.7446927644011</v>
       </c>
       <c r="T21" s="5" t="n">
-        <v>8.62220227286638</v>
+        <v>0.08622202272866382</v>
       </c>
       <c r="U21" s="5" t="n">
-        <v>11.963100707358</v>
+        <v>0.1196310070735798</v>
       </c>
       <c r="V21" s="5" t="n">
         <v>0.2</v>
       </c>
       <c r="W21" s="5" t="n">
-        <v>2.434261468154329</v>
+        <v>0.02443540055272938</v>
       </c>
       <c r="X21" s="5" t="n">
         <v>2</v>
@@ -8787,7 +8787,7 @@
         <v>373.4815881017068</v>
       </c>
       <c r="AF21" s="8" t="n">
-        <v>-32.2421280551856</v>
+        <v>-0.3169323888224952</v>
       </c>
       <c r="AG21" s="10" t="n">
         <v>0.918510983833304</v>
@@ -8844,7 +8844,7 @@
         <v>15.22000128194382</v>
       </c>
       <c r="AS21" s="8" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="AT21" s="5" t="n">
         <v>24.53886912626195</v>
@@ -8854,10 +8854,10 @@
         <v>0.623</v>
       </c>
       <c r="AW21" s="5" t="n">
-        <v>32.45072</v>
+        <v>32.316032</v>
       </c>
       <c r="AX21" s="5" t="n">
-        <v>5.988409</v>
+        <v>5.9635534</v>
       </c>
       <c r="AY21" s="5" t="n">
         <v>75</v>
@@ -8933,7 +8933,7 @@
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>47398080512</v>
+        <v>47500931072</v>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
@@ -8982,19 +8982,19 @@
         <v>6.97</v>
       </c>
       <c r="S22" s="5" t="n">
-        <v>42.88725182064557</v>
+        <v>42.93890821133753</v>
       </c>
       <c r="T22" s="5" t="n">
-        <v>8.870267856766869</v>
+        <v>0.08870267856766871</v>
       </c>
       <c r="U22" s="5" t="n">
-        <v>2.23342382333552</v>
+        <v>0.02233423823335517</v>
       </c>
       <c r="V22" s="5" t="n">
         <v>1.2</v>
       </c>
       <c r="W22" s="5" t="n">
-        <v>1.289839964156327</v>
+        <v>0.01288288260121594</v>
       </c>
       <c r="X22" s="5" t="n">
         <v>7.5</v>
@@ -9027,7 +9027,7 @@
         <v>140.009611591153</v>
       </c>
       <c r="AF22" s="8" t="n">
-        <v>-67.85990428020821</v>
+        <v>-0.6822416498645831</v>
       </c>
       <c r="AG22" s="10">
         <f>IF(H22="Fail","Not Eligible (Failed Gate)",IF(J22="","Pending Score",IF(J22&gt;=90,"10%",IF(J22&gt;=80,"7.5%",IF(J22&gt;=70,"5%","Watchlist only")))))</f>
@@ -9086,7 +9086,7 @@
         <v>3.4299999651009</v>
       </c>
       <c r="AS22" s="8" t="n">
-        <v>8.972</v>
+        <v>0.08971999999999999</v>
       </c>
       <c r="AT22" s="5" t="n">
         <v>40.8191287437763</v>
@@ -9096,10 +9096,10 @@
         <v>-0.195</v>
       </c>
       <c r="AW22" s="5" t="n">
-        <v>68.51895</v>
+        <v>68.66763</v>
       </c>
       <c r="AX22" s="5" t="n">
-        <v>6.093179</v>
+        <v>6.1064014</v>
       </c>
       <c r="AY22" s="5" t="n">
         <v>75</v>
@@ -9165,7 +9165,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n">
-        <v>1344131301376</v>
+        <v>1338356137984</v>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
@@ -9181,7 +9181,7 @@
         <v>33.3333333333333</v>
       </c>
       <c r="J23" s="10" t="n">
-        <v>30.92854221493596</v>
+        <v>30.97592967554693</v>
       </c>
       <c r="K23" s="5" t="n">
         <v>50</v>
@@ -9215,7 +9215,7 @@
       </c>
       <c r="S23" s="5" t="n"/>
       <c r="T23" s="5" t="n">
-        <v>14.9335779967161</v>
+        <v>0.1493357799671612</v>
       </c>
       <c r="U23" s="5" t="n">
         <v>10.26</v>
@@ -9224,7 +9224,7 @@
         <v>8.25</v>
       </c>
       <c r="W23" s="5" t="n">
-        <v>-0.4093271729665177</v>
+        <v>-0.004095271254601016</v>
       </c>
       <c r="X23" s="5" t="n">
         <v>10</v>
@@ -9248,22 +9248,22 @@
         </is>
       </c>
       <c r="AC23" s="6" t="n">
-        <v>718.3850880869193</v>
+        <v>719.0546800612697</v>
       </c>
       <c r="AD23" s="7" t="n">
         <v>423</v>
       </c>
       <c r="AE23" s="6" t="n">
-        <v>897.981360108649</v>
+        <v>898.8183500765871</v>
       </c>
       <c r="AF23" s="8" t="n">
-        <v>54.6427110746798</v>
+        <v>0.5487964837773465</v>
       </c>
       <c r="AG23" s="10" t="n">
-        <v>1.885728258453118</v>
+        <v>0.01884510916337611</v>
       </c>
       <c r="AH23" s="9" t="n">
-        <v>18857.28258453118</v>
+        <v>18845.10916337611</v>
       </c>
       <c r="AI23" s="5" t="inlineStr">
         <is>
@@ -9311,13 +9311,13 @@
         </is>
       </c>
       <c r="AR23" s="8" t="n">
-        <v>78.50000502068532</v>
+        <v>78.60000321726064</v>
       </c>
       <c r="AS23" s="8" t="n">
-        <v>16.12516180932</v>
+        <v>0.1612516180932</v>
       </c>
       <c r="AT23" s="5" t="n">
-        <v>11.43925299501464</v>
+        <v>11.43534796535098</v>
       </c>
       <c r="AU23" s="5" t="n">
         <v>3.91</v>
@@ -9326,10 +9326,10 @@
         <v>0.62</v>
       </c>
       <c r="AW23" s="5" t="n">
-        <v>5.1885347</v>
+        <v>5.159669</v>
       </c>
       <c r="AX23" s="5" t="n">
-        <v>1.0116062</v>
+        <v>1.0072597</v>
       </c>
       <c r="AY23" s="5" t="n">
         <v>50</v>
@@ -9405,7 +9405,7 @@
         </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>3543960125440</v>
+        <v>3522033614848</v>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
@@ -9421,7 +9421,7 @@
         <v>77</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>48.91786602675464</v>
+        <v>49.55755473969643</v>
       </c>
       <c r="K24" s="5" t="n">
         <v>80</v>
@@ -9454,19 +9454,19 @@
         <v>2.71</v>
       </c>
       <c r="S24" s="5" t="n">
-        <v>13.9288966962213</v>
+        <v>13.84323133970996</v>
       </c>
       <c r="T24" s="5" t="n">
-        <v>28.3911247262704</v>
+        <v>0.2839112472627043</v>
       </c>
       <c r="U24" s="5" t="n">
-        <v>33.1956468254828</v>
+        <v>0.3319564682548277</v>
       </c>
       <c r="V24" s="5" t="n">
         <v>0.03</v>
       </c>
       <c r="W24" s="5" t="n">
-        <v>4.566792358577275</v>
+        <v>0.04595052804849564</v>
       </c>
       <c r="X24" s="5" t="n">
         <v>9.869999999999999</v>
@@ -9499,13 +9499,13 @@
         <v>208.3374402345152</v>
       </c>
       <c r="AF24" s="8" t="n">
-        <v>-35.76532364111306</v>
+        <v>-0.3492534019981217</v>
       </c>
       <c r="AG24" s="10" t="n">
-        <v>5.96509215784039</v>
+        <v>0.06029956412748582</v>
       </c>
       <c r="AH24" s="9" t="n">
-        <v>59650.9215784039</v>
+        <v>60299.56412748582</v>
       </c>
       <c r="AI24" s="5" t="inlineStr">
         <is>
@@ -9556,7 +9556,7 @@
         <v>16.57999950878418</v>
       </c>
       <c r="AS24" s="8" t="n">
-        <v>5</v>
+        <v>0.05</v>
       </c>
       <c r="AT24" s="5" t="n">
         <v>12.56558746890924</v>
@@ -9568,10 +9568,10 @@
         <v>-0.081</v>
       </c>
       <c r="AW24" s="5" t="n">
-        <v>17.059711</v>
+        <v>16.954163</v>
       </c>
       <c r="AX24" s="5" t="n">
-        <v>4.887764</v>
+        <v>4.857523</v>
       </c>
       <c r="AY24" s="5" t="n">
         <v>100</v>
@@ -9647,7 +9647,7 @@
         </is>
       </c>
       <c r="F25" s="5" t="n">
-        <v>2022909542400</v>
+        <v>2024419360768</v>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
@@ -9696,19 +9696,19 @@
         <v>1.95</v>
       </c>
       <c r="S25" s="5" t="n">
-        <v>40.96722030456853</v>
+        <v>40.99775437878941</v>
       </c>
       <c r="T25" s="5" t="n">
-        <v>21.9728965763153</v>
+        <v>0.2197289657631528</v>
       </c>
       <c r="U25" s="5" t="n">
-        <v>18.2195155562466</v>
+        <v>0.1821951555624663</v>
       </c>
       <c r="V25" s="5" t="n">
         <v>0.05</v>
       </c>
       <c r="W25" s="5" t="n">
-        <v>1.74239487461802</v>
+        <v>0.01741097183677874</v>
       </c>
       <c r="X25" s="5" t="n">
         <v>15.6</v>
@@ -9741,13 +9741,13 @@
         <v>3807.357537937685</v>
       </c>
       <c r="AF25" s="8" t="n">
-        <v>-93.55944185877027</v>
+        <v>-0.9370389900378997</v>
       </c>
       <c r="AG25" s="10" t="n">
-        <v>4.35991269030482</v>
+        <v>0.04350432568290045</v>
       </c>
       <c r="AH25" s="9" t="n">
-        <v>43599.1269030482</v>
+        <v>43504.32568290045</v>
       </c>
       <c r="AI25" s="5" t="inlineStr">
         <is>
@@ -9798,7 +9798,7 @@
         <v>201.0399846555437</v>
       </c>
       <c r="AS25" s="8" t="n">
-        <v>15.4840062</v>
+        <v>0.154840062</v>
       </c>
       <c r="AT25" s="5" t="n">
         <v>18.9383084855635</v>
@@ -9810,10 +9810,10 @@
         <v>0.275</v>
       </c>
       <c r="AW25" s="5" t="n">
-        <v>36.656887</v>
+        <v>36.684242</v>
       </c>
       <c r="AX25" s="5" t="n">
-        <v>8.053834</v>
+        <v>8.059844999999999</v>
       </c>
       <c r="AY25" s="5" t="n">
         <v>100</v>
@@ -9889,7 +9889,7 @@
         </is>
       </c>
       <c r="F26" s="5" t="n">
-        <v>248079564800</v>
+        <v>247310647296</v>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
@@ -9938,19 +9938,19 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="S26" s="5" t="n">
-        <v/>
+        <v>17.07149716368106</v>
       </c>
       <c r="T26" s="5" t="n">
-        <v>9.91603175109184</v>
+        <v>0.09916031751091842</v>
       </c>
       <c r="U26" s="5" t="n">
-        <v>14.8115365111698</v>
+        <v>0.1481153651116976</v>
       </c>
       <c r="V26" s="5" t="n">
         <v>2.96</v>
       </c>
       <c r="W26" s="5" t="n">
-        <v/>
+        <v>-0.05903798618387057</v>
       </c>
       <c r="X26" s="5" t="n">
         <v>14</v>
@@ -9983,7 +9983,7 @@
         <v>730.2192303013911</v>
       </c>
       <c r="AF26" s="8" t="n">
-        <v>-112.073297406976</v>
+        <v>-1.114159605688296</v>
       </c>
       <c r="AG26" s="10">
         <f>IF(H26="Fail","Not Eligible (Failed Gate)",IF(J26="","Pending Score",IF(J26&gt;=90,"10%",IF(J26&gt;=80,"7.5%",IF(J26&gt;=70,"5%","Watchlist only")))))</f>
@@ -10042,7 +10042,7 @@
         <v>48.41000063208718</v>
       </c>
       <c r="AS26" s="8" t="n">
-        <v>10.5100006</v>
+        <v>0.105100006</v>
       </c>
       <c r="AT26" s="5" t="n">
         <v>15.08405763894632</v>
@@ -10052,10 +10052,10 @@
         <v>0.184</v>
       </c>
       <c r="AW26" s="5" t="n">
-        <v>31.989258</v>
+        <v>31.890106</v>
       </c>
       <c r="AX26" s="5" t="n">
-        <v>3.1633716</v>
+        <v>3.1535666</v>
       </c>
       <c r="AY26" s="5" t="n">
         <v>25</v>
@@ -10131,7 +10131,7 @@
         </is>
       </c>
       <c r="F27" s="5" t="n">
-        <v>1197219774464</v>
+        <v>1196185485312</v>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
@@ -10181,7 +10181,7 @@
       </c>
       <c r="S27" s="5" t="n"/>
       <c r="T27" s="5" t="n">
-        <v>12.2079359890616</v>
+        <v>0.1220793598906159</v>
       </c>
       <c r="U27" s="5" t="n">
         <v>15.27</v>
@@ -10190,7 +10190,7 @@
         <v>0.66</v>
       </c>
       <c r="W27" s="5" t="n">
-        <v>56.41939669927579</v>
+        <v>0.5655684786618228</v>
       </c>
       <c r="X27" s="5" t="n">
         <v>9.800000000000001</v>
@@ -10214,16 +10214,16 @@
         </is>
       </c>
       <c r="AC27" s="6" t="n">
-        <v>378.9407005294082</v>
+        <v>379.9526557318841</v>
       </c>
       <c r="AD27" s="7" t="n">
         <v>106</v>
       </c>
       <c r="AE27" s="6" t="n">
-        <v>473.6758756617602</v>
+        <v>474.9408196648551</v>
       </c>
       <c r="AF27" s="8" t="n">
-        <v>78.00816859113485</v>
+        <v>0.7808569074491329</v>
       </c>
       <c r="AG27" s="10" t="n">
         <v>0.565553626035105</v>
@@ -10277,13 +10277,13 @@
         </is>
       </c>
       <c r="AR27" s="8" t="n">
-        <v>16</v>
+        <v>16.39999964704074</v>
       </c>
       <c r="AS27" s="8" t="n">
-        <v>10.6308197597</v>
+        <v>0.106308197597</v>
       </c>
       <c r="AT27" s="5" t="n">
-        <v>29.60474222886002</v>
+        <v>28.95980607712531</v>
       </c>
       <c r="AU27" s="5" t="n">
         <v>2.97</v>
@@ -10292,10 +10292,10 @@
         <v>0.527</v>
       </c>
       <c r="AW27" s="5" t="n">
-        <v>6.510625</v>
+        <v>6.3463416</v>
       </c>
       <c r="AX27" s="5" t="n">
-        <v>0.7982926</v>
+        <v>0.79760295</v>
       </c>
       <c r="AY27" s="5" t="n">
         <v>60</v>
@@ -10371,7 +10371,7 @@
         </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>668463136768</v>
+        <v>663195090944</v>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
@@ -10420,19 +10420,19 @@
         <v>0.4</v>
       </c>
       <c r="S28" s="5" t="n">
-        <v>28.17657588361176</v>
+        <v>27.95377842858955</v>
       </c>
       <c r="T28" s="5" t="n">
-        <v>16.0702848996963</v>
+        <v>0.160702848996963</v>
       </c>
       <c r="U28" s="5" t="n">
-        <v>21.0890117731003</v>
+        <v>0.2108901177310025</v>
       </c>
       <c r="V28" s="5" t="n">
         <v>0.7</v>
       </c>
       <c r="W28" s="5" t="n">
-        <v>1.574819372466328</v>
+        <v>0.01587371011923637</v>
       </c>
       <c r="X28" s="5" t="n">
         <v>35.9</v>
@@ -10465,7 +10465,7 @@
         <v>719.5352351888428</v>
       </c>
       <c r="AF28" s="8" t="n">
-        <v>-109.8576867613299</v>
+        <v>-1.0820384141533</v>
       </c>
       <c r="AG28" s="10" t="n">
         <v>2.71436355448913</v>
@@ -10522,7 +10522,7 @@
         <v>44.50000166506629</v>
       </c>
       <c r="AS28" s="8" t="n">
-        <v>11.89214301142</v>
+        <v>0.1189214301142002</v>
       </c>
       <c r="AT28" s="5" t="n">
         <v>16.16933112783916</v>
@@ -10534,10 +10534,10 @@
         <v>0.23</v>
       </c>
       <c r="AW28" s="5" t="n">
-        <v>33.932583</v>
+        <v>33.66517</v>
       </c>
       <c r="AX28" s="5" t="n">
-        <v>5.317594</v>
+        <v>5.275687</v>
       </c>
       <c r="AY28" s="5" t="n">
         <v>100</v>
@@ -10603,7 +10603,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>494169686016</v>
+        <v>494891728896</v>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
@@ -10652,19 +10652,19 @@
         <v>0.5</v>
       </c>
       <c r="S29" s="5" t="n">
-        <v>26.84023772755777</v>
+        <v>26.8777516908077</v>
       </c>
       <c r="T29" s="5" t="n">
-        <v>35.0264780545114</v>
+        <v>0.3502647805451143</v>
       </c>
       <c r="U29" s="5" t="n">
-        <v>25.1812485600527</v>
+        <v>0.2518124856005272</v>
       </c>
       <c r="V29" s="5" t="n">
         <v>0.86</v>
       </c>
       <c r="W29" s="5" t="n">
-        <v>-3.361746055821881</v>
+        <v>-0.03357053981148208</v>
       </c>
       <c r="X29" s="5" t="n">
         <v>44</v>
@@ -10697,7 +10697,7 @@
         <v>156.8150114748871</v>
       </c>
       <c r="AF29" s="8" t="n">
-        <v>-598.2749863684812</v>
+        <v>-5.99295296850846</v>
       </c>
       <c r="AG29" s="10" t="n">
         <v>0.676806111126165</v>
@@ -10754,7 +10754,7 @@
         <v>35.06999859623924</v>
       </c>
       <c r="AS29" s="8" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT29" s="5" t="n">
         <v>4.471485927427633</v>
@@ -10764,10 +10764,10 @@
       </c>
       <c r="AV29" s="5" t="n"/>
       <c r="AW29" s="5" t="n">
-        <v>31.223269</v>
+        <v>31.26889</v>
       </c>
       <c r="AX29" s="5" t="n">
-        <v>11.451939</v>
+        <v>11.468672</v>
       </c>
       <c r="AY29" s="5" t="n">
         <v>50</v>
@@ -10833,7 +10833,7 @@
         </is>
       </c>
       <c r="F30" s="5" t="n">
-        <v>358072942592</v>
+        <v>357543411712</v>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
@@ -10849,7 +10849,7 @@
         <v>56.6666666666667</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>40.97818969485613</v>
+        <v>41.01815293415386</v>
       </c>
       <c r="K30" s="5" t="n">
         <v>92</v>
@@ -10883,7 +10883,7 @@
       </c>
       <c r="S30" s="5" t="n"/>
       <c r="T30" s="5" t="n">
-        <v>7.37602665529544</v>
+        <v>0.07376026655295435</v>
       </c>
       <c r="U30" s="5" t="n">
         <v>11.65</v>
@@ -10892,7 +10892,7 @@
         <v>0.05</v>
       </c>
       <c r="W30" s="5" t="n">
-        <v>5.153998094608051</v>
+        <v>0.05161844960189139</v>
       </c>
       <c r="X30" s="5" t="n">
         <v>26.4</v>
@@ -10925,13 +10925,13 @@
         <v>765.7036951392305</v>
       </c>
       <c r="AF30" s="8" t="n">
-        <v>20.52408733781215</v>
+        <v>0.2064162627692311</v>
       </c>
       <c r="AG30" s="10" t="n">
-        <v>2.998152182569755</v>
+        <v>0.02994550586164594</v>
       </c>
       <c r="AH30" s="9" t="n">
-        <v>29981.52182569755</v>
+        <v>29945.50586164594</v>
       </c>
       <c r="AI30" s="5" t="inlineStr">
         <is>
@@ -10982,7 +10982,7 @@
         <v>9.460000388628723</v>
       </c>
       <c r="AS30" s="8" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="AT30" s="5" t="n">
         <v>80.94119398934782</v>
@@ -10992,10 +10992,10 @@
         <v>0.204</v>
       </c>
       <c r="AW30" s="5" t="n">
-        <v>64.32875</v>
+        <v>64.23362</v>
       </c>
       <c r="AX30" s="5" t="n">
-        <v>4.706569</v>
+        <v>4.699609</v>
       </c>
       <c r="AY30" s="5" t="n">
         <v>60</v>
@@ -11061,7 +11061,7 @@
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>71626588160</v>
+        <v>70938116096</v>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
@@ -11077,7 +11077,7 @@
         <v>55</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>40.55107453992223</v>
+        <v>41.14684008331328</v>
       </c>
       <c r="K31" s="5" t="n">
         <v>40</v>
@@ -11110,19 +11110,19 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="S31" s="5" t="n">
-        <v>10.29938221862949</v>
+        <v>10.20814673752004</v>
       </c>
       <c r="T31" s="5" t="n">
-        <v>14.8502727479355</v>
+        <v>0.1485027274793545</v>
       </c>
       <c r="U31" s="5" t="n">
-        <v>20.1179226294038</v>
+        <v>0.2011792262940377</v>
       </c>
       <c r="V31" s="5" t="n">
         <v>1.81</v>
       </c>
       <c r="W31" s="5" t="n">
-        <v>-1.190746265621564</v>
+        <v>-0.01201388580158831</v>
       </c>
       <c r="X31" s="5" t="n">
         <v>28.5</v>
@@ -11155,7 +11155,7 @@
         <v>163.49721694134</v>
       </c>
       <c r="AF31" s="8" t="n">
-        <v>-20.9011405196704</v>
+        <v>-0.1973904122798537</v>
       </c>
       <c r="AG31" s="10" t="n">
         <v>0.681727293742978</v>
@@ -11212,7 +11212,7 @@
         <v>13.5899992875405</v>
       </c>
       <c r="AS31" s="8" t="n">
-        <v>21.336001</v>
+        <v>0.21336001</v>
       </c>
       <c r="AT31" s="5" t="n">
         <v>12.0307002900177</v>
@@ -11220,10 +11220,10 @@
       <c r="AU31" s="5" t="n"/>
       <c r="AV31" s="5" t="n"/>
       <c r="AW31" s="5" t="n">
-        <v>14.545254</v>
+        <v>14.405445</v>
       </c>
       <c r="AX31" s="5" t="n">
-        <v>2.2591374</v>
+        <v>2.2374227</v>
       </c>
       <c r="AY31" s="5" t="n">
         <v>25</v>
@@ -11289,7 +11289,7 @@
         </is>
       </c>
       <c r="F32" s="5" t="n">
-        <v>100881326080</v>
+        <v>99996622848</v>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
@@ -11338,19 +11338,19 @@
         <v>0.3</v>
       </c>
       <c r="S32" s="5" t="n">
-        <v>11.07908585865675</v>
+        <v>10.99038758088287</v>
       </c>
       <c r="T32" s="5" t="n">
-        <v>20.0820236161955</v>
+        <v>0.2008202361619554</v>
       </c>
       <c r="U32" s="5" t="n">
-        <v>25.1618290338693</v>
+        <v>0.2516182903386932</v>
       </c>
       <c r="V32" s="5" t="n">
         <v>0.5</v>
       </c>
       <c r="W32" s="5" t="n">
-        <v>8.938056513581477</v>
+        <v>0.09010191387221356</v>
       </c>
       <c r="X32" s="5" t="n">
         <v>89</v>
@@ -11383,7 +11383,7 @@
         <v>514.575831894859</v>
       </c>
       <c r="AF32" s="8" t="n">
-        <v>59.66969547796336</v>
+        <v>0.6002338484446511</v>
       </c>
       <c r="AG32" s="10" t="n">
         <v>7.01875492300514</v>
@@ -11440,7 +11440,7 @@
         <v>13.50999992578712</v>
       </c>
       <c r="AS32" s="8" t="n">
-        <v>21.6306065692</v>
+        <v>0.216306065692</v>
       </c>
       <c r="AT32" s="5" t="n">
         <v>38.0885145740088</v>
@@ -11452,10 +11452,10 @@
         <v>0.767</v>
       </c>
       <c r="AW32" s="5" t="n">
-        <v>15.361214</v>
+        <v>15.2265</v>
       </c>
       <c r="AX32" s="5" t="n">
-        <v>3.1007948</v>
+        <v>3.0736015</v>
       </c>
       <c r="AY32" s="5" t="n">
         <v>100</v>
@@ -11521,7 +11521,7 @@
         </is>
       </c>
       <c r="F33" s="5" t="n">
-        <v>751172911104</v>
+        <v>747128684544</v>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
@@ -11570,19 +11570,19 @@
         <v>0.28</v>
       </c>
       <c r="S33" s="5" t="n">
-        <v>9.267525717682156</v>
+        <v>9.221475974904068</v>
       </c>
       <c r="T33" s="5" t="n">
-        <v>21.8641785753694</v>
+        <v>0.2186417857536935</v>
       </c>
       <c r="U33" s="5" t="n">
-        <v>24.2510446894871</v>
+        <v>0.2425104468948705</v>
       </c>
       <c r="V33" s="5" t="n">
         <v>0.13</v>
       </c>
       <c r="W33" s="5" t="n">
-        <v>2.242899267214939</v>
+        <v>0.0225409974473215</v>
       </c>
       <c r="X33" s="5" t="n">
         <v>60.7</v>
@@ -11615,7 +11615,7 @@
         <v>94.71003782321692</v>
       </c>
       <c r="AF33" s="8" t="n">
-        <v>9.787809229387189</v>
+        <v>0.1027350220404171</v>
       </c>
       <c r="AG33" s="10" t="n">
         <v>5.28624892448139</v>
@@ -11672,7 +11672,7 @@
         <v>8.539999864063674</v>
       </c>
       <c r="AS33" s="8" t="n">
-        <v>13.7094084</v>
+        <v>0.137094084</v>
       </c>
       <c r="AT33" s="5" t="n">
         <v>11.09016836337435</v>
@@ -11684,10 +11684,10 @@
         <v>0.618</v>
       </c>
       <c r="AW33" s="5" t="n">
-        <v>10.004684</v>
+        <v>9.95082</v>
       </c>
       <c r="AX33" s="5" t="n">
-        <v>2.2012677</v>
+        <v>2.1894164</v>
       </c>
       <c r="AY33" s="5" t="n">
         <v>100</v>
@@ -11753,7 +11753,7 @@
         </is>
       </c>
       <c r="F34" s="5" t="n">
-        <v>62048972800</v>
+        <v>62044200960</v>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
@@ -11802,19 +11802,19 @@
         <v>0.38</v>
       </c>
       <c r="S34" s="5" t="n">
-        <v>17.36006367555787</v>
+        <v>17.35893328279718</v>
       </c>
       <c r="T34" s="5" t="n">
-        <v>24.4049537034222</v>
+        <v>0.2440495370342224</v>
       </c>
       <c r="U34" s="5" t="n">
-        <v>15.0990231811175</v>
+        <v>0.1509902318111746</v>
       </c>
       <c r="V34" s="5" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="W34" s="5" t="n">
-        <v>2.504237882250516</v>
+        <v>0.02504400955195555</v>
       </c>
       <c r="X34" s="5" t="n">
         <v>98</v>
@@ -11847,7 +11847,7 @@
         <v>579.5112172012732</v>
       </c>
       <c r="AF34" s="8" t="n">
-        <v>-12.08583729180883</v>
+        <v>-0.1207720933112128</v>
       </c>
       <c r="AG34" s="10" t="n">
         <v>0.390649115071915</v>
@@ -11904,7 +11904,7 @@
         <v>42.03000083406467</v>
       </c>
       <c r="AS34" s="8" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT34" s="5" t="n">
         <v>13.78803752560726</v>
@@ -11916,10 +11916,10 @@
         <v>0.661</v>
       </c>
       <c r="AW34" s="5" t="n">
-        <v>15.454437</v>
+        <v>15.453248</v>
       </c>
       <c r="AX34" s="5" t="n">
-        <v>3.7621703</v>
+        <v>3.7618809</v>
       </c>
       <c r="AY34" s="5" t="n">
         <v>100</v>
@@ -11985,7 +11985,7 @@
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>97757110272</v>
+        <v>96995786752</v>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
@@ -12034,19 +12034,19 @@
         <v>0.42</v>
       </c>
       <c r="S35" s="5" t="n">
-        <v>13.83342690526172</v>
+        <v>13.72844908326154</v>
       </c>
       <c r="T35" s="5" t="n">
-        <v>24.6688420964524</v>
+        <v>0.2466884209645236</v>
       </c>
       <c r="U35" s="5" t="n">
-        <v>23.0787036904442</v>
+        <v>0.2307870369044416</v>
       </c>
       <c r="V35" s="5" t="n">
         <v>0.1</v>
       </c>
       <c r="W35" s="5" t="n">
-        <v>7.633757073286334</v>
+        <v>0.07692130396184776</v>
       </c>
       <c r="X35" s="5" t="n">
         <v>36.7</v>
@@ -12079,7 +12079,7 @@
         <v>530.8830958541873</v>
       </c>
       <c r="AF35" s="8" t="n">
-        <v>55.25380222970112</v>
+        <v>0.5560227819633996</v>
       </c>
       <c r="AG35" s="10" t="n">
         <v>7.43043625290765</v>
@@ -12136,7 +12136,7 @@
         <v>16.09000050664367</v>
       </c>
       <c r="AS35" s="8" t="n">
-        <v>24.70821679857</v>
+        <v>0.2470821679857</v>
       </c>
       <c r="AT35" s="5" t="n">
         <v>32.99459887223041</v>
@@ -12148,10 +12148,10 @@
         <v>-0.247</v>
       </c>
       <c r="AW35" s="5" t="n">
-        <v>14.763828</v>
+        <v>14.6488495</v>
       </c>
       <c r="AX35" s="5" t="n">
-        <v>3.9686916</v>
+        <v>3.937784</v>
       </c>
       <c r="AY35" s="5" t="n">
         <v>100</v>
@@ -12217,7 +12217,7 @@
         </is>
       </c>
       <c r="F36" s="5" t="n">
-        <v>147534905344</v>
+        <v>147525713920</v>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
@@ -12266,19 +12266,19 @@
         <v>0.75</v>
       </c>
       <c r="S36" s="5" t="n">
-        <v>16.48774025815112</v>
+        <v>16.48669109985892</v>
       </c>
       <c r="T36" s="5" t="n">
-        <v>27.5407957769878</v>
+        <v>0.2754079577698776</v>
       </c>
       <c r="U36" s="5" t="n">
-        <v>29.2978587999153</v>
+        <v>0.2929785879991533</v>
       </c>
       <c r="V36" s="5" t="n">
         <v>0.13</v>
       </c>
       <c r="W36" s="5" t="n">
-        <v>5.222356559142746</v>
+        <v>0.0522268889257798</v>
       </c>
       <c r="X36" s="5" t="n">
         <v>23</v>
@@ -12311,7 +12311,7 @@
         <v>2231.128196759233</v>
       </c>
       <c r="AF36" s="8" t="n">
-        <v>28.14397656178221</v>
+        <v>0.2814845859917234</v>
       </c>
       <c r="AG36" s="5" t="n">
         <v>7.35604258074957</v>
@@ -12368,7 +12368,7 @@
         <v>78.4400067519467</v>
       </c>
       <c r="AS36" s="8" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT36" s="5" t="n">
         <v>28.4437556955537</v>
@@ -12380,10 +12380,10 @@
         <v>0.409</v>
       </c>
       <c r="AW36" s="5" t="n">
-        <v>20.43855</v>
+        <v>20.437277</v>
       </c>
       <c r="AX36" s="5" t="n">
-        <v>5.790129</v>
+        <v>5.789768</v>
       </c>
       <c r="AY36" s="5" t="n">
         <v>100</v>
@@ -12449,7 +12449,7 @@
         </is>
       </c>
       <c r="F37" s="5" t="n">
-        <v>82858508288</v>
+        <v>83210362880</v>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
@@ -12498,19 +12498,19 @@
         <v>0.21</v>
       </c>
       <c r="S37" s="5" t="n">
-        <v>11.28154961064244</v>
+        <v>11.33075839132673</v>
       </c>
       <c r="T37" s="5" t="n">
-        <v>21.7039608443092</v>
+        <v>0.2170396084430917</v>
       </c>
       <c r="U37" s="5" t="n">
-        <v>21.0666410064932</v>
+        <v>0.210666410064932</v>
       </c>
       <c r="V37" s="5" t="n">
         <v>0.1</v>
       </c>
       <c r="W37" s="5" t="n">
-        <v>1.96366644801301</v>
+        <v>0.01955138366463648</v>
       </c>
       <c r="X37" s="5" t="n">
         <v>13</v>
@@ -12543,7 +12543,7 @@
         <v>679.044095650445</v>
       </c>
       <c r="AF37" s="8" t="n">
-        <v>-35.24894861507928</v>
+        <v>-0.358232853960013</v>
       </c>
       <c r="AG37" s="5" t="n">
         <v>2.95492379755887</v>
@@ -12600,7 +12600,7 @@
         <v>75.4900018445521</v>
       </c>
       <c r="AS37" s="8" t="n">
-        <v>20.316037</v>
+        <v>0.20316037</v>
       </c>
       <c r="AT37" s="5" t="n">
         <v>8.99515294277977</v>
@@ -12612,10 +12612,10 @@
         <v>0.5590000000000001</v>
       </c>
       <c r="AW37" s="5" t="n">
-        <v>12.165851</v>
+        <v>12.217512</v>
       </c>
       <c r="AX37" s="5" t="n">
-        <v>2.641616</v>
+        <v>2.6528335</v>
       </c>
       <c r="AY37" s="5" t="n">
         <v>100</v>
@@ -12681,7 +12681,7 @@
         </is>
       </c>
       <c r="F38" s="5" t="n">
-        <v>276219166720</v>
+        <v>275910852608</v>
       </c>
       <c r="G38" s="5" t="n"/>
       <c r="H38" s="5" t="n"/>
@@ -12702,17 +12702,17 @@
       <c r="Q38" s="5" t="n"/>
       <c r="R38" s="5" t="n"/>
       <c r="S38" s="5" t="n">
-        <v/>
+        <v>108.0808983912088</v>
       </c>
       <c r="T38" s="5" t="n">
-        <v>2.46913580246914</v>
+        <v>0.02469135802469136</v>
       </c>
       <c r="U38" s="5" t="n">
-        <v>7.52895752895753</v>
+        <v>0.07528957528957529</v>
       </c>
       <c r="V38" s="5" t="n"/>
       <c r="W38" s="5" t="n">
-        <v/>
+        <v>0.01108245967263005</v>
       </c>
       <c r="X38" s="5" t="n"/>
       <c r="Y38" s="5" t="n"/>
@@ -12727,7 +12727,7 @@
         <v>88.78863258264307</v>
       </c>
       <c r="AF38" s="5" t="n">
-        <v>-505.370287125104</v>
+        <v>-5.046945249441269</v>
       </c>
       <c r="AG38" s="5" t="n"/>
       <c r="AH38" s="5" t="n"/>
@@ -12744,7 +12744,7 @@
         <v>1.220000029053024</v>
       </c>
       <c r="AS38" s="5" t="n">
-        <v>5</v>
+        <v>0.05</v>
       </c>
       <c r="AT38" s="5" t="n">
         <v>72.77756769069104</v>
@@ -12754,10 +12754,10 @@
         <v>1.417</v>
       </c>
       <c r="AW38" s="5" t="n">
-        <v>440.57376</v>
+        <v>440.08197</v>
       </c>
       <c r="AX38" s="5" t="n">
-        <v>11.555909</v>
+        <v>11.54301</v>
       </c>
       <c r="AY38" s="5" t="n">
         <v>75</v>
@@ -12823,7 +12823,7 @@
         </is>
       </c>
       <c r="F39" s="5" t="n">
-        <v>162603532288</v>
+        <v>162138882048</v>
       </c>
       <c r="G39" s="5" t="n"/>
       <c r="H39" s="5" t="n"/>
@@ -12844,17 +12844,17 @@
       <c r="Q39" s="5" t="n"/>
       <c r="R39" s="5" t="n"/>
       <c r="S39" s="5" t="n">
-        <v>41.45357366599928</v>
+        <v>41.33430413470917</v>
       </c>
       <c r="T39" s="5" t="n">
-        <v>12.733796156858</v>
+        <v>0.1273379615685802</v>
       </c>
       <c r="U39" s="5" t="n">
-        <v>14.3291157863763</v>
+        <v>0.1432911578637634</v>
       </c>
       <c r="V39" s="5" t="n"/>
       <c r="W39" s="5" t="n">
-        <v>0.7054095687522809</v>
+        <v>0.007074450177671826</v>
       </c>
       <c r="X39" s="5" t="n"/>
       <c r="Y39" s="5" t="n"/>
@@ -12869,13 +12869,13 @@
         <v>1477.478730938063</v>
       </c>
       <c r="AF39" s="5" t="n">
-        <v>-373.7124029904837</v>
+        <v>-3.723587456023126</v>
       </c>
       <c r="AG39" s="5" t="n">
-        <v>2.099347923341902</v>
+        <v>0.02094783135953154</v>
       </c>
       <c r="AH39" s="5" t="n">
-        <v>20993.47923341902</v>
+        <v>20947.83135953154</v>
       </c>
       <c r="AI39" s="5" t="n"/>
       <c r="AJ39" s="5" t="n"/>
@@ -12890,7 +12890,7 @@
         <v>145.300002673902</v>
       </c>
       <c r="AS39" s="5" t="n">
-        <v>12.345390480724</v>
+        <v>0.12345390480724</v>
       </c>
       <c r="AT39" s="5" t="n">
         <v>10.16847027486623</v>
@@ -12902,10 +12902,10 @@
         <v>0.667</v>
       </c>
       <c r="AW39" s="5" t="n">
-        <v>48.169304</v>
+        <v>48.03166</v>
       </c>
       <c r="AX39" s="5" t="n">
-        <v>6.121383</v>
+        <v>6.103891</v>
       </c>
       <c r="AY39" s="5" t="n">
         <v>100</v>
@@ -12971,7 +12971,7 @@
         </is>
       </c>
       <c r="F40" s="5" t="n">
-        <v>298218848256</v>
+        <v>289276887040</v>
       </c>
       <c r="G40" s="5" t="n"/>
       <c r="H40" s="5" t="n"/>
@@ -12992,17 +12992,17 @@
       <c r="Q40" s="5" t="n"/>
       <c r="R40" s="5" t="n"/>
       <c r="S40" s="5" t="n">
-        <v>266.2615414485506</v>
+        <v>258.2476311183406</v>
       </c>
       <c r="T40" s="5" t="n">
-        <v>24.0088525924023</v>
+        <v>0.2400885259240232</v>
       </c>
       <c r="U40" s="5" t="n">
-        <v>23.7089384932376</v>
+        <v>0.2370893849323763</v>
       </c>
       <c r="V40" s="5" t="n"/>
       <c r="W40" s="5" t="n">
-        <v>0.07212282541189514</v>
+        <v>0.0007436093250743501</v>
       </c>
       <c r="X40" s="5" t="n"/>
       <c r="Y40" s="5" t="n"/>
@@ -13017,13 +13017,13 @@
         <v>7.058060514374156</v>
       </c>
       <c r="AF40" s="5" t="n">
-        <v>-3042.222988147126</v>
+        <v>-29.48004470376458</v>
       </c>
       <c r="AG40" s="5" t="n">
-        <v>3.483817031414717</v>
+        <v>0.03476241877304771</v>
       </c>
       <c r="AH40" s="5" t="n">
-        <v>34838.17031414717</v>
+        <v>34762.41877304771</v>
       </c>
       <c r="AI40" s="5" t="n"/>
       <c r="AJ40" s="5" t="n"/>
@@ -13038,7 +13038,7 @@
         <v>0.8400000303002987</v>
       </c>
       <c r="AS40" s="5" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT40" s="5" t="n">
         <v>8.402452993302568</v>
@@ -13048,10 +13048,10 @@
         <v>0.288</v>
       </c>
       <c r="AW40" s="5" t="n">
-        <v>264.0238</v>
+        <v>256.10715</v>
       </c>
       <c r="AX40" s="5" t="n">
-        <v>66.06493</v>
+        <v>64.084</v>
       </c>
       <c r="AY40" s="5" t="n">
         <v>75</v>
@@ -13117,7 +13117,7 @@
         </is>
       </c>
       <c r="F41" s="5" t="n">
-        <v>229876105216</v>
+        <v>235098685440</v>
       </c>
       <c r="G41" s="5" t="n"/>
       <c r="H41" s="5" t="n"/>
@@ -13138,17 +13138,17 @@
       <c r="Q41" s="5" t="n"/>
       <c r="R41" s="5" t="n"/>
       <c r="S41" s="5" t="n">
-        <v>65.1115304503134</v>
+        <v>66.5827834185506</v>
       </c>
       <c r="T41" s="5" t="n">
-        <v>19.1442114239116</v>
+        <v>0.1914421142391158</v>
       </c>
       <c r="U41" s="5" t="n">
-        <v>23.8102744210007</v>
+        <v>0.2381027442100067</v>
       </c>
       <c r="V41" s="5" t="n"/>
       <c r="W41" s="5" t="n">
-        <v>-0.1043786440015852</v>
+        <v>-0.001020722311133983</v>
       </c>
       <c r="X41" s="5" t="n"/>
       <c r="Y41" s="5" t="n"/>
@@ -13163,13 +13163,13 @@
         <v>165.0669995877687</v>
       </c>
       <c r="AF41" s="5" t="n">
-        <v>-745.2931255093765</v>
+        <v>-7.644974486503838</v>
       </c>
       <c r="AG41" s="5" t="n">
-        <v>1.030216243623014</v>
+        <v>0.01027976158468816</v>
       </c>
       <c r="AH41" s="5" t="n">
-        <v>10302.16243623014</v>
+        <v>10279.76158468816</v>
       </c>
       <c r="AI41" s="5" t="n"/>
       <c r="AJ41" s="5" t="n"/>
@@ -13184,7 +13184,7 @@
         <v>15.47999878316759</v>
       </c>
       <c r="AS41" s="5" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT41" s="5" t="n">
         <v>10.66324286742692</v>
@@ -13192,10 +13192,10 @@
       <c r="AU41" s="5" t="n"/>
       <c r="AV41" s="5" t="n"/>
       <c r="AW41" s="5" t="n">
-        <v>90.135666</v>
+        <v>92.183464</v>
       </c>
       <c r="AX41" s="5" t="n">
-        <v>17.838833</v>
+        <v>18.244116</v>
       </c>
       <c r="AY41" s="5" t="n">
         <v>25</v>
@@ -13261,7 +13261,7 @@
         </is>
       </c>
       <c r="F42" s="5" t="n">
-        <v>88759902208</v>
+        <v>85371895808</v>
       </c>
       <c r="G42" s="5" t="n"/>
       <c r="H42" s="5" t="n"/>
@@ -13269,7 +13269,7 @@
         <v>87</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>53.9378447804087</v>
+        <v>57.59579075806278</v>
       </c>
       <c r="K42" s="5" t="n"/>
       <c r="L42" s="5" t="n">
@@ -13282,17 +13282,17 @@
       <c r="Q42" s="5" t="n"/>
       <c r="R42" s="5" t="n"/>
       <c r="S42" s="5" t="n">
-        <v>5.938837443454723</v>
+        <v>5.725560782348682</v>
       </c>
       <c r="T42" s="5" t="n">
-        <v>116.012608117596</v>
+        <v>1.160126081175961</v>
       </c>
       <c r="U42" s="5" t="n">
-        <v>112.12476266437</v>
+        <v>1.121247626643704</v>
       </c>
       <c r="V42" s="5" t="n"/>
       <c r="W42" s="5" t="n">
-        <v>-2.783507493571385</v>
+        <v>-0.02887192915307319</v>
       </c>
       <c r="X42" s="5" t="n"/>
       <c r="Y42" s="5" t="n"/>
@@ -13307,13 +13307,13 @@
         <v>213.7259425655053</v>
       </c>
       <c r="AF42" s="5" t="n">
-        <v>-27.97229794233861</v>
+        <v>-0.2308753763917598</v>
       </c>
       <c r="AG42" s="5" t="n">
-        <v>1.64430831229666</v>
+        <v>0.01752003855179687</v>
       </c>
       <c r="AH42" s="5" t="n">
-        <v>16443.0831229666</v>
+        <v>17520.03855179688</v>
       </c>
       <c r="AI42" s="5" t="n"/>
       <c r="AJ42" s="5" t="n"/>
@@ -13328,7 +13328,7 @@
         <v>49.20999701872088</v>
       </c>
       <c r="AS42" s="5" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT42" s="5" t="n">
         <v>4.343140470747924</v>
@@ -13338,10 +13338,10 @@
         <v>0.544</v>
       </c>
       <c r="AW42" s="5" t="n">
-        <v>5.558017</v>
+        <v>5.345865</v>
       </c>
       <c r="AX42" s="5" t="n">
-        <v>6.630385</v>
+        <v>6.3773003</v>
       </c>
       <c r="AY42" s="5" t="n">
         <v>25</v>
@@ -13407,7 +13407,7 @@
         </is>
       </c>
       <c r="F43" s="5" t="n">
-        <v>200479031296</v>
+        <v>200199290880</v>
       </c>
       <c r="G43" s="5" t="n"/>
       <c r="H43" s="5" t="n"/>
@@ -13428,17 +13428,17 @@
       <c r="Q43" s="5" t="n"/>
       <c r="R43" s="5" t="n"/>
       <c r="S43" s="5" t="n">
-        <v>39.53500261758846</v>
+        <v>39.48192598045726</v>
       </c>
       <c r="T43" s="5" t="n">
-        <v>24.8340395480226</v>
+        <v>0.248340395480226</v>
       </c>
       <c r="U43" s="5" t="n">
-        <v>34.095613921594</v>
+        <v>0.34095613921594</v>
       </c>
       <c r="V43" s="5" t="n"/>
       <c r="W43" s="5" t="n">
-        <v>1.192546512047195</v>
+        <v>0.01194149685066498</v>
       </c>
       <c r="X43" s="5" t="n"/>
       <c r="Y43" s="5" t="n"/>
@@ -13453,13 +13453,13 @@
         <v>2367.315286661589</v>
       </c>
       <c r="AF43" s="5" t="n">
-        <v>-172.460539428014</v>
+        <v>-1.720803619311376</v>
       </c>
       <c r="AG43" s="5" t="n">
-        <v>3.446175891723956</v>
+        <v>0.03438682583885345</v>
       </c>
       <c r="AH43" s="5" t="n">
-        <v>34461.75891723956</v>
+        <v>34386.82583885345</v>
       </c>
       <c r="AI43" s="5" t="n"/>
       <c r="AJ43" s="5" t="n"/>
@@ -13474,7 +13474,7 @@
         <v>112.9800007882326</v>
       </c>
       <c r="AS43" s="5" t="n">
-        <v>24.8410665</v>
+        <v>0.248410665</v>
       </c>
       <c r="AT43" s="5" t="n">
         <v>20.95340136892892</v>
@@ -13486,10 +13486,10 @@
         <v>0.504</v>
       </c>
       <c r="AW43" s="5" t="n">
-        <v>57.08975</v>
+        <v>57.01009</v>
       </c>
       <c r="AX43" s="5" t="n">
-        <v>14.158119</v>
+        <v>14.138363</v>
       </c>
       <c r="AY43" s="5" t="n">
         <v>100</v>
@@ -13555,7 +13555,7 @@
         </is>
       </c>
       <c r="F44" s="5" t="n">
-        <v>124590465024</v>
+        <v>123812986880</v>
       </c>
       <c r="G44" s="5" t="n"/>
       <c r="H44" s="5" t="n"/>
@@ -13576,17 +13576,17 @@
       <c r="Q44" s="5" t="n"/>
       <c r="R44" s="5" t="n"/>
       <c r="S44" s="5" t="n">
-        <v>33.1762805803174</v>
+        <v>32.97267765149531</v>
       </c>
       <c r="T44" s="5" t="n">
-        <v>12.2663351543699</v>
+        <v>0.1226633515436992</v>
       </c>
       <c r="U44" s="5" t="n">
-        <v>16.7170990190207</v>
+        <v>0.167170990190207</v>
       </c>
       <c r="V44" s="5" t="n"/>
       <c r="W44" s="5" t="n">
-        <v>1.652940640097758</v>
+        <v>0.01663147380328261</v>
       </c>
       <c r="X44" s="5" t="n"/>
       <c r="Y44" s="5" t="n"/>
@@ -13601,13 +13601,13 @@
         <v>152.5276559294702</v>
       </c>
       <c r="AF44" s="5" t="n">
-        <v>-89.11324522903648</v>
+        <v>-0.8793313137425312</v>
       </c>
       <c r="AG44" s="5" t="n">
-        <v>1.852863844409853</v>
+        <v>0.01848835007924014</v>
       </c>
       <c r="AH44" s="5" t="n">
-        <v>18528.63844409853</v>
+        <v>18488.35007924014</v>
       </c>
       <c r="AI44" s="5" t="n"/>
       <c r="AJ44" s="5" t="n"/>
@@ -13622,7 +13622,7 @@
         <v>6.869999928549142</v>
       </c>
       <c r="AS44" s="5" t="n">
-        <v>16.936001</v>
+        <v>0.16936001</v>
       </c>
       <c r="AT44" s="5" t="n">
         <v>22.20198776265942</v>
@@ -13630,10 +13630,10 @@
       <c r="AU44" s="5" t="n"/>
       <c r="AV44" s="5" t="n"/>
       <c r="AW44" s="5" t="n">
-        <v>41.9869</v>
+        <v>41.72489</v>
       </c>
       <c r="AX44" s="5" t="n">
-        <v>5.6793795</v>
+        <v>5.6439385</v>
       </c>
       <c r="AY44" s="5" t="n">
         <v>75</v>
@@ -13699,7 +13699,7 @@
         </is>
       </c>
       <c r="F45" s="5" t="n">
-        <v>100822802432</v>
+        <v>101257977856</v>
       </c>
       <c r="G45" s="5" t="n"/>
       <c r="H45" s="5" t="n"/>
@@ -13720,17 +13720,17 @@
       <c r="Q45" s="5" t="n"/>
       <c r="R45" s="5" t="n"/>
       <c r="S45" s="5" t="n">
-        <v>97.41802959327602</v>
+        <v>97.83844831996909</v>
       </c>
       <c r="T45" s="5" t="n">
-        <v>12.1485403825204</v>
+        <v>0.1214854038252044</v>
       </c>
       <c r="U45" s="5" t="n">
-        <v>13.7862603553448</v>
+        <v>0.1378626035534482</v>
       </c>
       <c r="V45" s="5" t="n"/>
       <c r="W45" s="5" t="n">
-        <v>-0.1306062996702164</v>
+        <v>-0.001300450751705609</v>
       </c>
       <c r="X45" s="5" t="n"/>
       <c r="Y45" s="5" t="n"/>
@@ -13745,13 +13745,13 @@
         <v>84.71506326656576</v>
       </c>
       <c r="AF45" s="5" t="n">
-        <v>-1376.832987851604</v>
+        <v>-13.83207296967102</v>
       </c>
       <c r="AG45" s="5" t="n">
-        <v>1.35477288146902</v>
+        <v>0.01351827085731597</v>
       </c>
       <c r="AH45" s="5" t="n">
-        <v>13547.7288146902</v>
+        <v>13518.27085731597</v>
       </c>
       <c r="AI45" s="5" t="n"/>
       <c r="AJ45" s="5" t="n"/>
@@ -13766,7 +13766,7 @@
         <v>10.46000048909762</v>
       </c>
       <c r="AS45" s="5" t="n">
-        <v>12.537592419424</v>
+        <v>0.12537592419424</v>
       </c>
       <c r="AT45" s="5" t="n">
         <v>8.098954423189843</v>
@@ -13778,10 +13778,10 @@
         <v>0.517</v>
       </c>
       <c r="AW45" s="5" t="n">
-        <v>119.608025</v>
+        <v>120.12428</v>
       </c>
       <c r="AX45" s="5" t="n">
-        <v>13.885682</v>
+        <v>13.945616</v>
       </c>
       <c r="AY45" s="5" t="n">
         <v>50</v>
@@ -13847,7 +13847,7 @@
         </is>
       </c>
       <c r="F46" s="5" t="n">
-        <v>200421539840</v>
+        <v>202717986816</v>
       </c>
       <c r="G46" s="5" t="n"/>
       <c r="H46" s="5" t="n"/>
@@ -13868,17 +13868,17 @@
       <c r="Q46" s="5" t="n"/>
       <c r="R46" s="5" t="n"/>
       <c r="S46" s="5" t="n">
-        <v>48.21308075490114</v>
+        <v>48.7518644518896</v>
       </c>
       <c r="T46" s="5" t="n">
-        <v>10.4292397668346</v>
+        <v>0.1042923976683463</v>
       </c>
       <c r="U46" s="5" t="n">
-        <v>12.3106339040082</v>
+        <v>0.123106339040082</v>
       </c>
       <c r="V46" s="5" t="n"/>
       <c r="W46" s="5" t="n">
-        <v>-0.6107271791074805</v>
+        <v>-0.006039776967828489</v>
       </c>
       <c r="X46" s="5" t="n"/>
       <c r="Y46" s="5" t="n"/>
@@ -13893,13 +13893,13 @@
         <v>463.1330233455365</v>
       </c>
       <c r="AF46" s="5" t="n">
-        <v>-593.4724664632258</v>
+        <v>-6.014183476992837</v>
       </c>
       <c r="AG46" s="5" t="n">
-        <v>1.070704752184298</v>
+        <v>0.01068376629487007</v>
       </c>
       <c r="AH46" s="5" t="n">
-        <v>10707.04752184298</v>
+        <v>10683.76629487007</v>
       </c>
       <c r="AI46" s="5" t="n"/>
       <c r="AJ46" s="5" t="n"/>
@@ -13914,7 +13914,7 @@
         <v>52.01999957369418</v>
       </c>
       <c r="AS46" s="5" t="n">
-        <v>10.43044942504</v>
+        <v>0.1043044942504</v>
       </c>
       <c r="AT46" s="5" t="n">
         <v>8.902980072001855</v>
@@ -13926,10 +13926,10 @@
         <v>0.767</v>
       </c>
       <c r="AW46" s="5" t="n">
-        <v>61.739716</v>
+        <v>62.447136</v>
       </c>
       <c r="AX46" s="5" t="n">
-        <v>6.4735045</v>
+        <v>6.547679</v>
       </c>
       <c r="AY46" s="5" t="n">
         <v>50</v>
@@ -13995,7 +13995,7 @@
         </is>
       </c>
       <c r="F47" s="5" t="n">
-        <v>131477848064</v>
+        <v>130693496832</v>
       </c>
       <c r="G47" s="5" t="n"/>
       <c r="H47" s="5" t="n"/>
@@ -14016,17 +14016,17 @@
       <c r="Q47" s="5" t="n"/>
       <c r="R47" s="5" t="n"/>
       <c r="S47" s="5" t="n">
-        <v>41.44157348761654</v>
+        <v>41.1951729739256</v>
       </c>
       <c r="T47" s="5" t="n">
-        <v>21.7141969730283</v>
+        <v>0.2171419697302833</v>
       </c>
       <c r="U47" s="5" t="n">
-        <v>33.1299784936568</v>
+        <v>0.3312997849365675</v>
       </c>
       <c r="V47" s="5" t="n"/>
       <c r="W47" s="5" t="n">
-        <v>0.5170918220771115</v>
+        <v>0.005201847012031642</v>
       </c>
       <c r="X47" s="5" t="n"/>
       <c r="Y47" s="5" t="n"/>
@@ -14041,13 +14041,13 @@
         <v>350.2017712597467</v>
       </c>
       <c r="AF47" s="5" t="n">
-        <v>-388.2328247083111</v>
+        <v>-3.853202180806207</v>
       </c>
       <c r="AG47" s="5" t="n">
-        <v>3.83856851484306</v>
+        <v>0.03830221994977259</v>
       </c>
       <c r="AH47" s="5" t="n">
-        <v>38385.6851484306</v>
+        <v>38302.21994977258</v>
       </c>
       <c r="AI47" s="5" t="n"/>
       <c r="AJ47" s="5" t="n"/>
@@ -14062,7 +14062,7 @@
         <v>27.27000024370429</v>
       </c>
       <c r="AS47" s="5" t="n">
-        <v>25</v>
+        <v>0.25</v>
       </c>
       <c r="AT47" s="5" t="n">
         <v>12.84201581443883</v>
@@ -14070,10 +14070,10 @@
       <c r="AU47" s="5" t="n"/>
       <c r="AV47" s="5" t="n"/>
       <c r="AW47" s="5" t="n">
-        <v>62.698936</v>
+        <v>62.324898</v>
       </c>
       <c r="AX47" s="5" t="n">
-        <v>14.14882</v>
+        <v>14.064413</v>
       </c>
       <c r="AY47" s="5" t="n">
         <v>75</v>
@@ -14139,7 +14139,7 @@
         </is>
       </c>
       <c r="F48" s="5" t="n">
-        <v>122639581184</v>
+        <v>122434224128</v>
       </c>
       <c r="G48" s="5" t="n"/>
       <c r="H48" s="5" t="n"/>
@@ -14160,17 +14160,17 @@
       <c r="Q48" s="5" t="n"/>
       <c r="R48" s="5" t="n"/>
       <c r="S48" s="5" t="n">
-        <v>34.26941402000426</v>
+        <v>34.21478615875719</v>
       </c>
       <c r="T48" s="5" t="n">
-        <v>9.39062982401976</v>
+        <v>0.0939062982401976</v>
       </c>
       <c r="U48" s="5" t="n">
-        <v>13.1553253661353</v>
+        <v>0.1315532536613533</v>
       </c>
       <c r="V48" s="5" t="n"/>
       <c r="W48" s="5" t="n">
-        <v>-0.2208412315203548</v>
+        <v>-0.002211938300751769</v>
       </c>
       <c r="X48" s="5" t="n"/>
       <c r="Y48" s="5" t="n"/>
@@ -14185,13 +14185,13 @@
         <v>108.7869892008311</v>
       </c>
       <c r="AF48" s="5" t="n">
-        <v>-476.4016493207716</v>
+        <v>-4.754364603696723</v>
       </c>
       <c r="AG48" s="5" t="n">
-        <v>1.004310405206515</v>
+        <v>0.01002126649278733</v>
       </c>
       <c r="AH48" s="5" t="n">
-        <v>10043.10405206515</v>
+        <v>10021.26649278733</v>
       </c>
       <c r="AI48" s="5" t="n"/>
       <c r="AJ48" s="5" t="n"/>
@@ -14206,7 +14206,7 @@
         <v>12.4399996428993</v>
       </c>
       <c r="AS48" s="5" t="n">
-        <v>9.427155600000001</v>
+        <v>0.09427155600000001</v>
       </c>
       <c r="AT48" s="5" t="n">
         <v>8.744934823217932</v>
@@ -14218,10 +14218,10 @@
         <v>0.201</v>
       </c>
       <c r="AW48" s="5" t="n">
-        <v>50.40595</v>
+        <v>50.321545</v>
       </c>
       <c r="AX48" s="5" t="n">
-        <v>4.7339892</v>
+        <v>4.726062</v>
       </c>
       <c r="AY48" s="5" t="n">
         <v>50</v>
@@ -14287,7 +14287,7 @@
         </is>
       </c>
       <c r="F49" s="5" t="n">
-        <v>75173560320</v>
+        <v>76599205888</v>
       </c>
       <c r="G49" s="5" t="n"/>
       <c r="H49" s="5" t="n"/>
@@ -14308,17 +14308,17 @@
       <c r="Q49" s="5" t="n"/>
       <c r="R49" s="5" t="n"/>
       <c r="S49" s="5" t="n">
-        <v>37.08120887484041</v>
+        <v>37.7631600692453</v>
       </c>
       <c r="T49" s="5" t="n">
-        <v>7.77052744996233</v>
+        <v>0.07770527449962328</v>
       </c>
       <c r="U49" s="5" t="n">
-        <v>8.932029485017109</v>
+        <v>0.08932029485017115</v>
       </c>
       <c r="V49" s="5" t="n"/>
       <c r="W49" s="5" t="n">
-        <v>-4.590691641634156</v>
+        <v>-0.04507790008338203</v>
       </c>
       <c r="X49" s="5" t="n"/>
       <c r="Y49" s="5" t="n"/>
@@ -14333,13 +14333,13 @@
         <v>583.7955157052062</v>
       </c>
       <c r="AF49" s="5" t="n">
-        <v>-297.4165504161837</v>
+        <v>-3.049534359893538</v>
       </c>
       <c r="AG49" s="5" t="n">
-        <v>0.612044282061547</v>
+        <v>0.006107134631015041</v>
       </c>
       <c r="AH49" s="5" t="n">
-        <v>6120.44282061547</v>
+        <v>6107.13463101504</v>
       </c>
       <c r="AI49" s="5" t="n"/>
       <c r="AJ49" s="5" t="n"/>
@@ -14354,7 +14354,7 @@
         <v>55.54999547478594</v>
       </c>
       <c r="AS49" s="5" t="n">
-        <v>6.3833084</v>
+        <v>0.063833084</v>
       </c>
       <c r="AT49" s="5" t="n">
         <v>10.50937021971568</v>
@@ -14366,10 +14366,10 @@
         <v>0.764</v>
       </c>
       <c r="AW49" s="5" t="n">
-        <v>41.76598</v>
+        <v>42.55806</v>
       </c>
       <c r="AX49" s="5" t="n">
-        <v>3.8034554</v>
+        <v>3.8755867</v>
       </c>
       <c r="AY49" s="5" t="n">
         <v>50</v>
@@ -14395,7 +14395,7 @@
       <c r="BF49" s="5" t="n"/>
       <c r="BG49" s="5" t="inlineStr">
         <is>
-          <t>Significantly Overvalued</t>
+          <t>Extreme Premium</t>
         </is>
       </c>
       <c r="BH49" s="5" t="inlineStr">
@@ -14435,7 +14435,7 @@
         </is>
       </c>
       <c r="F50" s="5" t="n">
-        <v>172049842176</v>
+        <v>171850465280</v>
       </c>
       <c r="G50" s="5" t="n"/>
       <c r="H50" s="5" t="n"/>
@@ -14456,17 +14456,17 @@
       <c r="Q50" s="5" t="n"/>
       <c r="R50" s="5" t="n"/>
       <c r="S50" s="5" t="n">
-        <v>59.71266234237316</v>
+        <v>59.64391652449276</v>
       </c>
       <c r="T50" s="5" t="n">
-        <v>14.6793722546181</v>
+        <v>0.1467937225461808</v>
       </c>
       <c r="U50" s="5" t="n">
-        <v>19.7337102705853</v>
+        <v>0.1973371027058525</v>
       </c>
       <c r="V50" s="5" t="n"/>
       <c r="W50" s="5" t="n">
-        <v>1.755932138263332</v>
+        <v>0.01757956032702554</v>
       </c>
       <c r="X50" s="5" t="n"/>
       <c r="Y50" s="5" t="n"/>
@@ -14481,13 +14481,13 @@
         <v>729.9092314283693</v>
       </c>
       <c r="AF50" s="5" t="n">
-        <v>-148.2637459528874</v>
+        <v>-1.479760389463751</v>
       </c>
       <c r="AG50" s="5" t="n">
-        <v>2.60006262975344</v>
+        <v>0.02594409096591886</v>
       </c>
       <c r="AH50" s="5" t="n">
-        <v>26000.62629753441</v>
+        <v>25944.09096591886</v>
       </c>
       <c r="AI50" s="5" t="n"/>
       <c r="AJ50" s="5" t="n"/>
@@ -14502,7 +14502,7 @@
         <v>20.53000168977967</v>
       </c>
       <c r="AS50" s="5" t="n">
-        <v>14.258650936024</v>
+        <v>0.14258650936024</v>
       </c>
       <c r="AT50" s="5" t="n">
         <v>35.55329914409982</v>
@@ -14514,10 +14514,10 @@
         <v>0.504</v>
       </c>
       <c r="AW50" s="5" t="n">
-        <v>88.265945</v>
+        <v>88.16365999999999</v>
       </c>
       <c r="AX50" s="5" t="n">
-        <v>13.090276</v>
+        <v>13.075106</v>
       </c>
       <c r="AY50" s="5" t="n">
         <v>100</v>

</xml_diff>